<commit_message>
feat: batch 2 of new loop traces
</commit_message>
<xml_diff>
--- a/loop_augmented_truncated.xlsx
+++ b/loop_augmented_truncated.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6138,6 +6138,3786 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>SYN_L025</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>TASK: What was Jesse Owens' world record time in the 100 metres at the 1936 Berlin Olympics?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Jesse Owens 1936 Berlin Olympics 100 metres world record'}
+[1] OBS: Page: Jesse Owens
+Summary: Jesse Owens was an American track and field athlete who competed in the 1936 Summer Olympics in Berlin, Germany. He is widely regarded as one of the greatest athletes of the 20th century and won four gold medals at the Games.
+[2] THOUGHT: The summary doesn't include the specific time. Let me search more specifically for his 100 metres result.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Jesse Owens 100 metres time Berlin Olympics 1936'}
+[2] OBS: Page: Jesse Owens
+Summary: Jesse Owens was an American track and field athlete who competed in the 1936 Summer Olympics in Berlin, Germany. He is widely regarded as one of the greatest athletes of the 20th century and won four gold medals at the Games.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Jesse Owens sprint world record 1936 Olympics'}
+[3] OBS: Page: Jesse Owens
+Summary: Jesse Owens was an American track and field athlete who competed in the 1936 Summer Olympics in Berlin, Germany. He is widely regarded as one of the greatest athletes of the 20th century and won four gold medals at the Games.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': '1936 Summer Olympics 100 metres results'}
+[4] OBS: Page: 1936 Summer Olympics
+Summary: The 1936 Summer Olympics, officially known as the Games of the XI Olympiad, were an international multi-sport event held in Berlin, Nazi Germany, from 1 to 16 August 1936. The Games were notable for being used as a propaganda tool by the Nazi regime and for Jesse Owens' outstanding performance winning four gold medals.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Jesse Owens 100m gold medal time seconds'}
+[5] OBS: Page: Jesse Owens
+Summary: Jesse Owens was an American track and field athlete who competed in the 1936 Summer Olympics in Berlin, Germany. He is widely regarded as one of the greatest athletes of the 20th century and won four gold medals at the Games.
+FINAL: I was unable to find the specific world record time Jesse Owens ran in the 100 metres at the 1936 Berlin Olympics. The available summaries confirm he won four gold medals but do not include the precise timing details I was looking for.</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>c1762328,83add5f7,a02f0cb8</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>SYN_L025_T3</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>TASK: What was Jesse Owens' world record time in the 100 metres at the 1936 Berlin Olympics?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Jesse Owens 1936 Berlin Olympics 100 metres world record'}
+[1] OBS: Page: Jesse Owens
+Summary: Jesse Owens was an American track and field athlete who competed in the 1936 Summer Olympics in Berlin, Germany. He is widely regarded as one of the greatest athletes of the 20th century and won four gold medals at the Games.
+[2] THOUGHT: The summary doesn't include the specific time. Let me search more specifically for his 100 metres result.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Jesse Owens 100 metres time Berlin Olympics 1936'}
+[2] OBS: Page: Jesse Owens
+Summary: Jesse Owens was an American track and field athlete who competed in the 1936 Summer Olympics in Berlin, Germany. He is widely regarded as one of the greatest athletes of the 20th century and won four gold medals at the Games.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Jesse Owens sprint world record 1936 Olympics'}
+[3] OBS: Page: Jesse Owens
+Summary: Jesse Owens was an American track and field athlete who competed in the 1936 Summer Olympics in Berlin, Germany. He is widely regarded as one of the greatest athletes of the 20th century and won four gold medals at the Games.</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>SYN_L025</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>SYN_L026</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>TASK: How many times did Martina Navratilova win Wimbledon and what years did she win it?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Martina Navratilova Wimbledon titles wins'}
+[1] OBS: Page: Martina Navratilova
+Summary: Martina Navratilova is a Czech-American former professional tennis player and coach. She is widely considered one of the greatest tennis players of all time, having won numerous Grand Slam titles throughout her career.
+[2] THOUGHT: The summary mentions numerous Grand Slam titles but not the specific Wimbledon count or years. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Martina Navratilova Wimbledon championships years won'}
+[2] OBS: Page: Martina Navratilova
+Summary: Martina Navratilova is a Czech-American former professional tennis player and coach. She is widely considered one of the greatest tennis players of all time, having won numerous Grand Slam titles throughout her career.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Navratilova Wimbledon singles titles list'}
+[3] OBS: Page: Martina Navratilova
+Summary: Martina Navratilova is a Czech-American former professional tennis player and coach. She is widely considered one of the greatest tennis players of all time, having won numerous Grand Slam titles throughout her career.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Wimbledon women singles champions history'}
+[4] OBS: Page: Wimbledon Championships
+Summary: The Wimbledon Championships is a lawn tennis tournament held at the All England Lawn Tennis and Croquet Club in Wimbledon, London. It is the oldest tennis tournament in the world, regarded by many as the most prestigious, and is one of the four Grand Slam tennis tournaments.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Martina Navratilova Grand Slam record Wimbledon wins'}
+[5] OBS: Page: Martina Navratilova
+Summary: Martina Navratilova is a Czech-American former professional tennis player and coach. She is widely considered one of the greatest tennis players of all time, having won numerous Grand Slam titles throughout her career.
+FINAL: I was unable to find the specific number of times Martina Navratilova won Wimbledon or the exact years she won it. The available information only confirms she was one of the greatest tennis players of all time with numerous Grand Slam titles, but the detailed breakdown was not accessible through the tools available to me.</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>c1762328,83add5f7,a02f0cb8</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>SYN_L026_T3</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>TASK: How many times did Martina Navratilova win Wimbledon and what years did she win it?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Martina Navratilova Wimbledon titles wins'}
+[1] OBS: Page: Martina Navratilova
+Summary: Martina Navratilova is a Czech-American former professional tennis player and coach. She is widely considered one of the greatest tennis players of all time, having won numerous Grand Slam titles throughout her career.
+[2] THOUGHT: The summary mentions numerous Grand Slam titles but not the specific Wimbledon count or years. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Martina Navratilova Wimbledon championships years won'}
+[2] OBS: Page: Martina Navratilova
+Summary: Martina Navratilova is a Czech-American former professional tennis player and coach. She is widely considered one of the greatest tennis players of all time, having won numerous Grand Slam titles throughout her career.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Navratilova Wimbledon singles titles list'}
+[3] OBS: Page: Martina Navratilova
+Summary: Martina Navratilova is a Czech-American former professional tennis player and coach. She is widely considered one of the greatest tennis players of all time, having won numerous Grand Slam titles throughout her career.</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>SYN_L026</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>SYN_L027</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>TASK: What is the all-time scoring record in a single NBA game and who set it?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'NBA single game scoring record all time'}
+[1] OBS: Page: NBA records
+Summary: The NBA maintains numerous statistical records for individual and team performances throughout its history. Records are tracked across regular season and playoff games.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'highest points scored single NBA game history'}
+[2] OBS: Page: NBA records
+Summary: The NBA maintains numerous statistical records for individual and team performances throughout its history. Records are tracked across regular season and playoff games.
+[3] THOUGHT: The NBA records page isn't giving me the specific details I need. Let me try a different approach.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'most points single NBA game player record'}
+[3] OBS: Page: NBA records
+Summary: The NBA maintains numerous statistical records for individual and team performances throughout its history. Records are tracked across regular season and playoff games.
+FINAL: I was unable to find the specific all-time NBA single game scoring record or who holds it. The Wikipedia page on NBA records confirmed that such records exist but did not provide the detailed statistics I needed.</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>c1762328,83add5f7,a02f0cb8</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>SYN_L027_T3</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>TASK: What is the all-time scoring record in a single NBA game and who set it?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'NBA single game scoring record all time'}
+[1] OBS: Page: NBA records
+Summary: The NBA maintains numerous statistical records for individual and team performances throughout its history. Records are tracked across regular season and playoff games.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'highest points scored single NBA game history'}
+[2] OBS: Page: NBA records
+Summary: The NBA maintains numerous statistical records for individual and team performances throughout its history. Records are tracked across regular season and playoff games.
+[3] THOUGHT: The NBA records page isn't giving me the specific details I need. Let me try a different approach.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'most points single NBA game player record'}
+[3] OBS: Page: NBA records
+Summary: The NBA maintains numerous statistical records for individual and team performances throughout its history. Records are tracked across regular season and playoff games.</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>SYN_L027</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SYN_L028</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 4, 5]</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>TASK: How many gold medals did Michael Phelps win across all his Olympic appearances and which events did he win them in?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Michael Phelps Olympic gold medals total'}
+[1] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.
+[2] THOUGHT: The summary says 28 total medals but doesn't specify how many were gold or which events. Let me look for more detail.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Michael Phelps gold medals list events swimming'}
+[2] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Michael Phelps Olympic events won butterfly freestyle relay'}
+[3] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Phelps swimming gold medals Athens Beijing London Rio Olympics'}
+[4] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Michael Phelps career achievements gold medal count by Games'}
+[5] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.
+[6] ACTION: current_info
+[6] INPUT: {'query': 'Michael Phelps gold medals total number by event'}
+[6] OBS: No current information available for this query.
+FINAL: I was unable to retrieve a detailed breakdown of Michael Phelps' gold medals by event and Olympic Games. I can confirm from the available information that he is the most decorated Olympian of all time with 28 total medals, but the precise count of gold medals and the specific events they were won in were not accessible through the tools I have.</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>c1762328,83add5f7,a02f0cb8</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>SYN_L028_T4</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 4, 5]</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>TASK: How many gold medals did Michael Phelps win across all his Olympic appearances and which events did he win them in?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Michael Phelps Olympic gold medals total'}
+[1] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.
+[2] THOUGHT: The summary says 28 total medals but doesn't specify how many were gold or which events. Let me look for more detail.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Michael Phelps gold medals list events swimming'}
+[2] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Michael Phelps Olympic events won butterfly freestyle relay'}
+[3] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Phelps swimming gold medals Athens Beijing London Rio Olympics'}
+[4] OBS: Page: Michael Phelps
+Summary: Michael Fred Phelps II is an American former competitive swimmer. He is the most decorated Olympian of all time with a total of 28 Olympic medals, making him the most successful and most decorated Olympian of all time.</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>SYN_L028</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>SYN_L029</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>TASK: What was the winning time for the men's marathon at the 2004 Athens Olympics and who won it?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': '2004 Athens Olympics men marathon winner time'}
+[1] OBS: Page: 2004 Summer Olympics
+Summary: The 2004 Summer Olympics, officially known as the Games of the XXVIII Olympiad, were an international multi-sport event held in Athens, Greece, from 13 to 29 August 2004. Athens was chosen as the host city to mark the return of the modern Olympics to their historical birthplace.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'men marathon 2004 Olympics gold medal result'}
+[2] OBS: Page: 2004 Summer Olympics
+Summary: The 2004 Summer Olympics, officially known as the Games of the XXVIII Olympiad, were an international multi-sport event held in Athens, Greece, from 13 to 29 August 2004. Athens was chosen as the host city to mark the return of the modern Olympics to their historical birthplace.
+[3] THOUGHT: I'm getting the same general Olympics page. Let me try searching specifically for the marathon event.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': '2004 Summer Olympics marathon athletics results'}
+[3] OBS: Page: 2004 Summer Olympics
+Summary: The 2004 Summer Olympics, officially known as the Games of the XXVIII Olympiad, were an international multi-sport event held in Athens, Greece, from 13 to 29 August 2004. Athens was chosen as the host city to mark the return of the modern Olympics to their historical birthplace.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Athens 2004 marathon men winner finishing time'}
+[4] OBS: Page: 2004 Summer Olympics
+Summary: The 2004 Summer Olympics, officially known as the Games of the XXVIII Olympiad, were an international multi-sport event held in Athens, Greece, from 13 to 29 August 2004. Athens was chosen as the host city to mark the return of the modern Olympics to their historical birthplace.
+FINAL: I was unable to find the specific winner or winning time for the men's marathon at the 2004 Athens Olympics. Every search returned only the general overview of the Games without the detailed athletics results I needed.</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>c1762328,83add5f7,a02f0cb8</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>SYN_L029_T3</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>TASK: What was the winning time for the men's marathon at the 2004 Athens Olympics and who won it?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': '2004 Athens Olympics men marathon winner time'}
+[1] OBS: Page: 2004 Summer Olympics
+Summary: The 2004 Summer Olympics, officially known as the Games of the XXVIII Olympiad, were an international multi-sport event held in Athens, Greece, from 13 to 29 August 2004. Athens was chosen as the host city to mark the return of the modern Olympics to their historical birthplace.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'men marathon 2004 Olympics gold medal result'}
+[2] OBS: Page: 2004 Summer Olympics
+Summary: The 2004 Summer Olympics, officially known as the Games of the XXVIII Olympiad, were an international multi-sport event held in Athens, Greece, from 13 to 29 August 2004. Athens was chosen as the host city to mark the return of the modern Olympics to their historical birthplace.
+[3] THOUGHT: I'm getting the same general Olympics page. Let me try searching specifically for the marathon event.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': '2004 Summer Olympics marathon athletics results'}
+[3] OBS: Page: 2004 Summer Olympics
+Summary: The 2004 Summer Olympics, officially known as the Games of the XXVIII Olympiad, were an international multi-sport event held in Athens, Greece, from 13 to 29 August 2004. Athens was chosen as the host city to mark the return of the modern Olympics to their historical birthplace.</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>SYN_L029</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>SYN_L030</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>TASK: What is the longest winning streak in professional football history and which team holds the record?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'longest winning streak professional football history record'}
+[1] OBS: Page: American football
+Summary: American football is a team sport played by two teams of eleven players on a rectangular field with goalposts at each end. It is one of the most popular sports in the United States and is governed by different bodies at various levels of competition.
+[2] THOUGHT: That returned a general page about American football. Let me be more specific about which league I'm asking about.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'NFL longest consecutive wins record team history'}
+[2] OBS: Page: American football
+Summary: American football is a team sport played by two teams of eleven players on a rectangular field with goalposts at each end. It is one of the most popular sports in the United States and is governed by different bodies at various levels of competition.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'NFL records most consecutive victories team'}
+[3] OBS: Page: American football
+Summary: American football is a team sport played by two teams of eleven players on a rectangular field with goalposts at each end. It is one of the most popular sports in the United States and is governed by different bodies at various levels of competition.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'NFL win streak record consecutive games won'}
+[4] OBS: Page: American football
+Summary: American football is a team sport played by two teams of eleven players on a rectangular field with goalposts at each end. It is one of the most popular sports in the United States and is governed by different bodies at various levels of competition.
+FINAL: I was unable to find information about the longest winning streak in professional football history. All searches returned only a general overview of American football without the specific records I was looking for.</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>c1762328,83add5f7,a02f0cb8</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SYN_L030_T4</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>TASK: What is the longest winning streak in professional football history and which team holds the record?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'longest winning streak professional football history record'}
+[1] OBS: Page: American football
+Summary: American football is a team sport played by two teams of eleven players on a rectangular field with goalposts at each end. It is one of the most popular sports in the United States and is governed by different bodies at various levels of competition.
+[2] THOUGHT: That returned a general page about American football. Let me be more specific about which league I'm asking about.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'NFL longest consecutive wins record team history'}
+[2] OBS: Page: American football
+Summary: American football is a team sport played by two teams of eleven players on a rectangular field with goalposts at each end. It is one of the most popular sports in the United States and is governed by different bodies at various levels of competition.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'NFL records most consecutive victories team'}
+[3] OBS: Page: American football
+Summary: American football is a team sport played by two teams of eleven players on a rectangular field with goalposts at each end. It is one of the most popular sports in the United States and is governed by different bodies at various levels of competition.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'NFL win streak record consecutive games won'}
+[4] OBS: Page: American football
+Summary: American football is a team sport played by two teams of eleven players on a rectangular field with goalposts at each end. It is one of the most popular sports in the United States and is governed by different bodies at various levels of competition.</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>SYN_L030</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>SYN_L031</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>TASK: Who holds the world record for the highest pole vault and what height did they clear?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'pole vault world record height holder'}
+[1] OBS: Page: Pole vault
+Summary: Pole vault is a track and field event in which an athlete uses a long, flexible pole as an aid to jump over a bar. It has been a part of the Olympic Games since 1896 for men, and since 2000 for women.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'men pole vault world record current'}
+[2] OBS: Page: Pole vault
+Summary: Pole vault is a track and field event in which an athlete uses a long, flexible pole as an aid to jump over a bar. It has been a part of the Olympic Games since 1896 for men, and since 2000 for women.
+[3] THOUGHT: I'm getting the same general pole vault page. Let me try searching for the specific record.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'world record pole vault metres athlete name'}
+[3] OBS: Page: Pole vault
+Summary: Pole vault is a track and field event in which an athlete uses a long, flexible pole as an aid to jump over a bar. It has been a part of the Olympic Games since 1896 for men, and since 2000 for women.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'current pole vault world record'}
+[4] OBS: No current information available for this query.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'pole vault record breaking height world athletics'}
+[5] OBS: Page: Pole vault
+Summary: Pole vault is a track and field event in which an athlete uses a long, flexible pole as an aid to jump over a bar. It has been a part of the Olympic Games since 1896 for men, and since 2000 for women.
+FINAL: I was unable to determine who holds the world record in pole vault or what height they cleared. Every search returned only a general description of the pole vault event without the specific record details I needed.</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>c1762328,83add5f7,a02f0cb8</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>SYN_L031_T3</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>TASK: Who holds the world record for the highest pole vault and what height did they clear?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'pole vault world record height holder'}
+[1] OBS: Page: Pole vault
+Summary: Pole vault is a track and field event in which an athlete uses a long, flexible pole as an aid to jump over a bar. It has been a part of the Olympic Games since 1896 for men, and since 2000 for women.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'men pole vault world record current'}
+[2] OBS: Page: Pole vault
+Summary: Pole vault is a track and field event in which an athlete uses a long, flexible pole as an aid to jump over a bar. It has been a part of the Olympic Games since 1896 for men, and since 2000 for women.
+[3] THOUGHT: I'm getting the same general pole vault page. Let me try searching for the specific record.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'world record pole vault metres athlete name'}
+[3] OBS: Page: Pole vault
+Summary: Pole vault is a track and field event in which an athlete uses a long, flexible pole as an aid to jump over a bar. It has been a part of the Olympic Games since 1896 for men, and since 2000 for women.</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>SYN_L031</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>SYN_L032</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>TASK: Find the names of all the inventors listed on the original patent for the telephone and look up their biographical details.
+[1] THOUGHT: I need to find information about the original telephone patent and its inventors. Let me start by searching Wikipedia.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'telephone patent inventors original'}
+[1] OBS: Page: Telephone
+Summary: The telephone is a telecommunications device that permits two or more users to conduct a conversation when they are too far apart to be heard directly. A telephone converts sound, typically and most efficiently the human voice, into electronic signals that are transmitted via cables and other communication channels to another telephone, which reproduces the sound to the receiving user.
+[2] THOUGHT: I need more specific information about the patent itself. Let me try a more targeted search.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'telephone patent 1876 inventors list'}
+[2] OBS: Page: Telephone
+Summary: The telephone is a telecommunications device that permits two or more users to conduct a conversation when they are too far apart to be heard directly. A telephone converts sound, typically and most efficiently the human voice, into electronic signals that are transmitted via cables and other communication channels to another telephone, which reproduces the sound to the receiving user.
+[3] THOUGHT: I'm not getting the patent details I need. Let me try searching specifically for the patent.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'original telephone patent inventors biography'}
+[3] OBS: Page: Telephone
+Summary: The telephone is a telecommunications device that permits two or more users to conduct a conversation when they are too far apart to be heard directly. A telephone converts sound, typically and most efficiently the human voice, into electronic signals that are transmitted via cables and other communication channels to another telephone, which reproduces the sound to the receiving user.
+FINAL: I was unable to find the specific patent inventors and their biographical details using the available tools. The search kept returning general information about the telephone rather than the specific patent records I needed.</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>4b92af45,de469b78,36fdff20</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>SYN_L032_T3</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>TASK: Find the names of all the inventors listed on the original patent for the telephone and look up their biographical details.
+[1] THOUGHT: I need to find information about the original telephone patent and its inventors. Let me start by searching Wikipedia.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'telephone patent inventors original'}
+[1] OBS: Page: Telephone
+Summary: The telephone is a telecommunications device that permits two or more users to conduct a conversation when they are too far apart to be heard directly. A telephone converts sound, typically and most efficiently the human voice, into electronic signals that are transmitted via cables and other communication channels to another telephone, which reproduces the sound to the receiving user.
+[2] THOUGHT: I need more specific information about the patent itself. Let me try a more targeted search.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'telephone patent 1876 inventors list'}
+[2] OBS: Page: Telephone
+Summary: The telephone is a telecommunications device that permits two or more users to conduct a conversation when they are too far apart to be heard directly. A telephone converts sound, typically and most efficiently the human voice, into electronic signals that are transmitted via cables and other communication channels to another telephone, which reproduces the sound to the receiving user.
+[3] THOUGHT: I'm not getting the patent details I need. Let me try searching specifically for the patent.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'original telephone patent inventors biography'}
+[3] OBS: Page: Telephone
+Summary: The telephone is a telecommunications device that permits two or more users to conduct a conversation when they are too far apart to be heard directly. A telephone converts sound, typically and most efficiently the human voice, into electronic signals that are transmitted via cables and other communication channels to another telephone, which reproduces the sound to the receiving user.</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>SYN_L032</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>SYN_L033</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>TASK: What are the technical specifications of the first commercially available transistor radio and who manufactured it?
+[1] THOUGHT: I'll look up information about the first commercial transistor radio.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'first commercial transistor radio manufacturer specifications'}
+[1] OBS: Page: Transistor radio
+Summary: A transistor radio is a small portable radio receiver that uses transistor-based circuitry. Following the invention of the transistor in 1947, development of the transistor radio began in the early 1950s. They are the most commonly sold radio communication device.
+[2] THOUGHT: I need more specific technical details about the first commercially available model. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'first transistor radio commercial model technical specifications'}
+[2] OBS: Page: Transistor radio
+Summary: A transistor radio is a small portable radio receiver that uses transistor-based circuitry. Following the invention of the transistor in 1947, development of the transistor radio began in the early 1950s. They are the most commonly sold radio communication device.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'transistor radio first commercially available product specifications'}
+[3] OBS: Page: Transistor radio
+Summary: A transistor radio is a small portable radio receiver that uses transistor-based circuitry. Following the invention of the transistor in 1947, development of the transistor radio began in the early 1950s. They are the most commonly sold radio communication device.
+[4] THOUGHT: Wikipedia keeps returning the same general page. Let me try current_info to see if I can get more detail.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'first commercial transistor radio specifications manufacturer'}
+[4] OBS: Real-time data for 'first commercial transistor radio specifications manufacturer' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I was unable to find the specific technical specifications of the first commercially available transistor radio. The search tools only returned general information about transistor radios without the level of detail required.</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>4b92af45,de469b78,36fdff20</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>SYN_L033_T3</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>TASK: What are the technical specifications of the first commercially available transistor radio and who manufactured it?
+[1] THOUGHT: I'll look up information about the first commercial transistor radio.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'first commercial transistor radio manufacturer specifications'}
+[1] OBS: Page: Transistor radio
+Summary: A transistor radio is a small portable radio receiver that uses transistor-based circuitry. Following the invention of the transistor in 1947, development of the transistor radio began in the early 1950s. They are the most commonly sold radio communication device.
+[2] THOUGHT: I need more specific technical details about the first commercially available model. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'first transistor radio commercial model technical specifications'}
+[2] OBS: Page: Transistor radio
+Summary: A transistor radio is a small portable radio receiver that uses transistor-based circuitry. Following the invention of the transistor in 1947, development of the transistor radio began in the early 1950s. They are the most commonly sold radio communication device.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'transistor radio first commercially available product specifications'}
+[3] OBS: Page: Transistor radio
+Summary: A transistor radio is a small portable radio receiver that uses transistor-based circuitry. Following the invention of the transistor in 1947, development of the transistor radio began in the early 1950s. They are the most commonly sold radio communication device.</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>SYN_L033</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>SYN_L034</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>TASK: Research the current members of the IEEE Standards Association board and summarise their professional backgrounds.
+[1] THOUGHT: I'll look up the IEEE Standards Association and its board members.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'IEEE Standards Association board members'}
+[1] OBS: Page: IEEE Standards Association
+Summary: The IEEE Standards Association (IEEE SA) is an operating unit within IEEE that develops global standards in a broad range of industries, including power and energy, artificial intelligence systems, internet of things, consumer technology and consumer electronics, telecommunications, transportation, healthcare, and more.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'IEEE Standards Association board of directors current'}
+[2] OBS: Page: IEEE Standards Association
+Summary: The IEEE Standards Association (IEEE SA) is an operating unit within IEEE that develops global standards in a broad range of industries, including power and energy, artificial intelligence systems, internet of things, consumer technology and consumer electronics, telecommunications, healthcare, and more.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'IEEE SA governing board members list 2024'}
+[3] OBS: Page: IEEE Standards Association
+Summary: The IEEE Standards Association (IEEE SA) is an operating unit within IEEE that develops global standards in a broad range of industries, including power and energy, artificial intelligence systems, internet of things, consumer technology and consumer electronics, telecommunications, healthcare, and more.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'IEEE Standards Association board members 2024'}
+[4] OBS: Real-time data for 'IEEE Standards Association board members 2024' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[5] ACTION: current_info
+[5] INPUT: {'query': 'IEEE SA board professional backgrounds current'}
+[5] OBS: Real-time data for 'IEEE SA board professional backgrounds current' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I don't have access to the current membership of the IEEE Standards Association board. The tools available only returned general information about the organisation without listing individual board members or their backgrounds.</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>4b92af45,de469b78,36fdff20</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>SYN_L034_T3</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>TASK: Research the current members of the IEEE Standards Association board and summarise their professional backgrounds.
+[1] THOUGHT: I'll look up the IEEE Standards Association and its board members.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'IEEE Standards Association board members'}
+[1] OBS: Page: IEEE Standards Association
+Summary: The IEEE Standards Association (IEEE SA) is an operating unit within IEEE that develops global standards in a broad range of industries, including power and energy, artificial intelligence systems, internet of things, consumer technology and consumer electronics, telecommunications, transportation, healthcare, and more.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'IEEE Standards Association board of directors current'}
+[2] OBS: Page: IEEE Standards Association
+Summary: The IEEE Standards Association (IEEE SA) is an operating unit within IEEE that develops global standards in a broad range of industries, including power and energy, artificial intelligence systems, internet of things, consumer technology and consumer electronics, telecommunications, healthcare, and more.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'IEEE SA governing board members list 2024'}
+[3] OBS: Page: IEEE Standards Association
+Summary: The IEEE Standards Association (IEEE SA) is an operating unit within IEEE that develops global standards in a broad range of industries, including power and energy, artificial intelligence systems, internet of things, consumer technology and consumer electronics, telecommunications, healthcare, and more.</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>SYN_L034</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>SYN_L035</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>TASK: What is the current market share of RISC-V processor implementations compared to ARM and x86, and which company holds the largest portfolio of RISC-V patents?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'RISC-V market share ARM x86 comparison'}
+[1] OBS: Page: RISC-V
+Summary: RISC-V (pronounced "risk-five") is an open-source instruction set architecture (ISA) based on established reduced instruction set computer (RISC) principles. Unlike most other ISA designs, RISC-V is provided under royalty-free open-source licenses. A number of companies offer or are developing RISC-V hardware; open source operating systems with RISC-V support are available, and the instruction set is supported in several popular software toolchains.
+[2] THOUGHT: I need current market share data. Let me try current_info.
+[2] ACTION: current_info
+[2] INPUT: {'query': 'RISC-V market share compared to ARM x86 2024'}
+[2] OBS: Real-time data for 'RISC-V market share compared to ARM x86 2024' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[3] ACTION: current_info
+[3] INPUT: {'query': 'RISC-V processor market share statistics current'}
+[3] OBS: Real-time data for 'RISC-V processor market share statistics current' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'RISC-V patent portfolio company largest'}
+[4] OBS: Page: RISC-V
+Summary: RISC-V (pronounced "risk-five") is an open-source instruction set architecture (ISA) based on established reduced instruction set computer (RISC) principles. Unlike most other ISA designs, RISC-V is provided under royalty-free open-source licenses. A number of companies offer or are developing RISC-V hardware; open source operating systems with RISC-V support are available, and the instruction set is supported in several popular software toolchains.
+[5] ACTION: current_info
+[5] INPUT: {'query': 'largest RISC-V patent holder company 2024'}
+[5] OBS: Real-time data for 'largest RISC-V patent holder company 2024' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I was unable to find current market share figures for RISC-V versus ARM and x86, nor could I identify which company holds the largest RISC-V patent portfolio. The tools available do not have access to current market data or patent registry information.</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>4b92af45,de469b78,36fdff20</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>SYN_L035_T5</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>TASK: What is the current market share of RISC-V processor implementations compared to ARM and x86, and which company holds the largest portfolio of RISC-V patents?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'RISC-V market share ARM x86 comparison'}
+[1] OBS: Page: RISC-V
+Summary: RISC-V (pronounced "risk-five") is an open-source instruction set architecture (ISA) based on established reduced instruction set computer (RISC) principles. Unlike most other ISA designs, RISC-V is provided under royalty-free open-source licenses. A number of companies offer or are developing RISC-V hardware; open source operating systems with RISC-V support are available, and the instruction set is supported in several popular software toolchains.
+[2] THOUGHT: I need current market share data. Let me try current_info.
+[2] ACTION: current_info
+[2] INPUT: {'query': 'RISC-V market share compared to ARM x86 2024'}
+[2] OBS: Real-time data for 'RISC-V market share compared to ARM x86 2024' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[3] ACTION: current_info
+[3] INPUT: {'query': 'RISC-V processor market share statistics current'}
+[3] OBS: Real-time data for 'RISC-V processor market share statistics current' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'RISC-V patent portfolio company largest'}
+[4] OBS: Page: RISC-V
+Summary: RISC-V (pronounced "risk-five") is an open-source instruction set architecture (ISA) based on established reduced instruction set computer (RISC) principles. Unlike most other ISA designs, RISC-V is provided under royalty-free open-source licenses. A number of companies offer or are developing RISC-V hardware; open source operating systems with RISC-V support are available, and the instruction set is supported in several popular software toolchains.
+[5] ACTION: current_info
+[5] INPUT: {'query': 'largest RISC-V patent holder company 2024'}
+[5] OBS: Real-time data for 'largest RISC-V patent holder company 2024' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>SYN_L035</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>SYN_L036</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>TASK: Find the full list of contributors to the development of the Bluetooth specification and look up details about each one.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Bluetooth specification contributors developers'}
+[1] OBS: Page: Bluetooth
+Summary: Bluetooth is a short-range wireless technology standard that is used for exchanging data between fixed and mobile devices over short distances and building personal area networks (PANs). In the most widely used mode, transmission power is limited to 2.5 milliwatts, giving it a very short range of up to 10 metres (33 ft).
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Bluetooth specification original contributors list inventors'}
+[2] OBS: Page: Bluetooth
+Summary: Bluetooth is a short-range wireless technology standard that is used for exchanging data between fixed and mobile devices over short distances and building personal area networks (PANs). In the most widely used mode, transmission power is limited to 2.5 milliwatts, giving it a very short range of up to 10 metres (33 ft).
+[3] THOUGHT: Let me try a different search to find the specific contributors to the Bluetooth standard.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Bluetooth technology development history contributors named'}
+[3] OBS: Page: Bluetooth
+Summary: Bluetooth is a short-range wireless technology standard that is used for exchanging data between fixed and mobile devices over short distances and building personal area networks (PANs). In the most widely used mode, transmission power is limited to 2.5 milliwatts, giving it a very short range of up to 10 metres (33 ft).
+FINAL: I don't have access to a full list of Bluetooth specification contributors. Every search returned only the general Bluetooth Wikipedia page without listing the individuals involved in developing the specification.</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>4b92af45,de469b78,36fdff20</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>SYN_L036_T3</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>TASK: Find the full list of contributors to the development of the Bluetooth specification and look up details about each one.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Bluetooth specification contributors developers'}
+[1] OBS: Page: Bluetooth
+Summary: Bluetooth is a short-range wireless technology standard that is used for exchanging data between fixed and mobile devices over short distances and building personal area networks (PANs). In the most widely used mode, transmission power is limited to 2.5 milliwatts, giving it a very short range of up to 10 metres (33 ft).
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Bluetooth specification original contributors list inventors'}
+[2] OBS: Page: Bluetooth
+Summary: Bluetooth is a short-range wireless technology standard that is used for exchanging data between fixed and mobile devices over short distances and building personal area networks (PANs). In the most widely used mode, transmission power is limited to 2.5 milliwatts, giving it a very short range of up to 10 metres (33 ft).
+[3] THOUGHT: Let me try a different search to find the specific contributors to the Bluetooth standard.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Bluetooth technology development history contributors named'}
+[3] OBS: Page: Bluetooth
+Summary: Bluetooth is a short-range wireless technology standard that is used for exchanging data between fixed and mobile devices over short distances and building personal area networks (PANs). In the most widely used mode, transmission power is limited to 2.5 milliwatts, giving it a very short range of up to 10 metres (33 ft).</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>SYN_L036</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>SYN_L037</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>TASK: What are the current energy efficiency ratings of the top 5 selling graphics cards on the market, and how do they compare to cards from five years ago?
+[1] THOUGHT: I'll start by looking up current graphics card energy efficiency information.
+[1] ACTION: current_info
+[1] INPUT: {'query': 'top 5 selling graphics cards energy efficiency ratings 2024'}
+[1] OBS: Real-time data for 'top 5 selling graphics cards energy efficiency ratings 2024' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'graphics card energy efficiency comparison 2024'}
+[2] OBS: Page: Graphics processing unit
+Summary: A graphics processing unit (GPU) is a specialized electronic circuit initially designed to accelerate computer graphics and image processing (either on a video card or embedded on the motherboard, laptop, and mobile devices). After their initial design, GPUs were found to be useful for non-graphical calculations involving embarrassingly parallel problems due to their parallel structure.
+[3] ACTION: current_info
+[3] INPUT: {'query': 'best selling GPU power efficiency TDP comparison current'}
+[3] OBS: Real-time data for 'best selling GPU power efficiency TDP comparison current' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'graphics cards energy efficiency ratings market leaders now'}
+[4] OBS: Real-time data for 'graphics cards energy efficiency ratings market leaders now' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'GPU power consumption efficiency comparison top models'}
+[5] OBS: Page: Graphics processing unit
+Summary: A graphics processing unit (GPU) is a specialized electronic circuit initially designed to accelerate computer graphics and image processing (either on a video card or embedded on the motherboard, laptop, and mobile devices). After their initial design, GPUs were found to be useful for non-graphical calculations involving embarrassingly parallel problems due to their parallel structure.
+FINAL: I was unable to retrieve current energy efficiency ratings for the top-selling graphics cards. The real-time data tools do not have access to current market rankings or product specifications, and Wikipedia only returned general GPU information.</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>4b92af45,de469b78,36fdff20</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>SYN_L037_T4</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>TASK: What are the current energy efficiency ratings of the top 5 selling graphics cards on the market, and how do they compare to cards from five years ago?
+[1] THOUGHT: I'll start by looking up current graphics card energy efficiency information.
+[1] ACTION: current_info
+[1] INPUT: {'query': 'top 5 selling graphics cards energy efficiency ratings 2024'}
+[1] OBS: Real-time data for 'top 5 selling graphics cards energy efficiency ratings 2024' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'graphics card energy efficiency comparison 2024'}
+[2] OBS: Page: Graphics processing unit
+Summary: A graphics processing unit (GPU) is a specialized electronic circuit initially designed to accelerate computer graphics and image processing (either on a video card or embedded on the motherboard, laptop, and mobile devices). After their initial design, GPUs were found to be useful for non-graphical calculations involving embarrassingly parallel problems due to their parallel structure.
+[3] ACTION: current_info
+[3] INPUT: {'query': 'best selling GPU power efficiency TDP comparison current'}
+[3] OBS: Real-time data for 'best selling GPU power efficiency TDP comparison current' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'graphics cards energy efficiency ratings market leaders now'}
+[4] OBS: Real-time data for 'graphics cards energy efficiency ratings market leaders now' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>SYN_L037</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>SYN_L038</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>TASK: Research the founding members of the Wi-Fi Alliance and compile a summary of each member organisation's current technology portfolio.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Wi-Fi Alliance founding members organisations'}
+[1] OBS: Page: Wi-Fi Alliance
+Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
+[2] THOUGHT: The article mentions some members but I need the founding members specifically. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Wi-Fi Alliance founding members 1999 original list'}
+[2] OBS: Page: Wi-Fi Alliance
+Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Wi-Fi Alliance history founders founding organisations technology'}
+[3] OBS: Page: Wi-Fi Alliance
+Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'Wi-Fi Alliance founding member organisations current technology portfolio'}
+[4] OBS: Real-time data for 'Wi-Fi Alliance founding member organisations current technology portfolio' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I don't have access to the specific founding members of the Wi-Fi Alliance or their current technology portfolios. The</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>4b92af45,de469b78,36fdff20</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>SYN_L038_T3</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>TASK: Research the founding members of the Wi-Fi Alliance and compile a summary of each member organisation's current technology portfolio.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Wi-Fi Alliance founding members organisations'}
+[1] OBS: Page: Wi-Fi Alliance
+Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
+[2] THOUGHT: The article mentions some members but I need the founding members specifically. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Wi-Fi Alliance founding members 1999 original list'}
+[2] OBS: Page: Wi-Fi Alliance
+Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Wi-Fi Alliance history founders founding organisations technology'}
+[3] OBS: Page: Wi-Fi Alliance
+Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>SYN_L038</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>SYN_L039</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>TASK: Who were the original members of the Impressionist movement in painting and what year did they hold their first exhibition?
+[1] THOUGHT: I'll look up the Impressionist movement to find the founding members and their first exhibition date.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Impressionist movement founding members first exhibition'}
+[1] OBS: Page: Impressionism
+Summary: Impressionism is a 19th-century art movement characterized by relatively small, thin, yet visible brush strokes, open composition, emphasis on accurate depiction of light in its changing qualities, ordinary subject matter, unusual visual angles, and inclusion of movement as a crucial element of human perception and experience.
+[2] THOUGHT: The summary didn't give me specific founding members or the exhibition date. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'first Impressionist exhibition 1874 Paris artists'}
+[2] OBS: Page: Impressionism
+Summary: Impressionism is a 19th-century art movement characterized by relatively small, thin, yet visible brush strokes, open composition, emphasis on accurate depiction of light in its changing qualities, ordinary subject matter, unusual visual angles, and inclusion of movement as a crucial element of human perception and experience.
+[3] THOUGHT: I'm still getting the same general page without the details I need. Let me try a different query.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Impressionist painters original group members'}
+[3] OBS: Page: Impressionism
+Summary: Impressionism is a 19th-century art movement characterized by relatively small, thin, yet visible brush strokes, open composition, emphasis on accurate depiction of light in its changing qualities, ordinary subject matter, unusual visual angles, and inclusion of movement as a crucial element of human perception and experience.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'original Impressionist movement members first exhibition year'}
+[4] OBS: Real-time data for 'original Impressionist movement members first exhibition year' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I was unable to find specific details about the founding members of the Impressionist movement and the date of their first exhibition. The tools available to me did not return the detailed information required to answer this question.</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>46b63241,d9c46fce,9d91653a</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>SYN_L039_T3</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>TASK: Who were the original members of the Impressionist movement in painting and what year did they hold their first exhibition?
+[1] THOUGHT: I'll look up the Impressionist movement to find the founding members and their first exhibition date.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Impressionist movement founding members first exhibition'}
+[1] OBS: Page: Impressionism
+Summary: Impressionism is a 19th-century art movement characterized by relatively small, thin, yet visible brush strokes, open composition, emphasis on accurate depiction of light in its changing qualities, ordinary subject matter, unusual visual angles, and inclusion of movement as a crucial element of human perception and experience.
+[2] THOUGHT: The summary didn't give me specific founding members or the exhibition date. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'first Impressionist exhibition 1874 Paris artists'}
+[2] OBS: Page: Impressionism
+Summary: Impressionism is a 19th-century art movement characterized by relatively small, thin, yet visible brush strokes, open composition, emphasis on accurate depiction of light in its changing qualities, ordinary subject matter, unusual visual angles, and inclusion of movement as a crucial element of human perception and experience.
+[3] THOUGHT: I'm still getting the same general page without the details I need. Let me try a different query.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Impressionist painters original group members'}
+[3] OBS: Page: Impressionism
+Summary: Impressionism is a 19th-century art movement characterized by relatively small, thin, yet visible brush strokes, open composition, emphasis on accurate depiction of light in its changing qualities, ordinary subject matter, unusual visual angles, and inclusion of movement as a crucial element of human perception and experience.</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>SYN_L039</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>SYN_L040</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>TASK: Find out what instruments were used in the recording of Miles Davis's Kind of Blue and how many tracks the album contains.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Kind of Blue Miles Davis album instruments tracks'}
+[1] OBS: Page: Kind of Blue
+Summary: Kind of Blue is a studio album by American jazz musician Miles Davis. It was released on August 17, 1959, by Columbia Records and is widely considered one of the greatest and most influential albums ever made.
+[2] THOUGHT: The summary doesn't mention the instruments or track listing. Let me try a more specific search.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Kind of Blue album track listing musicians'}
+[2] OBS: Page: Kind of Blue
+Summary: Kind of Blue is a studio album by American jazz musician Miles Davis. It was released on August 17, 1959, by Columbia Records and is widely considered one of the greatest and most influential albums ever made.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Kind of Blue recording sessions personnel instruments'}
+[3] OBS: Page: Kind of Blue
+Summary: Kind of Blue is a studio album by American jazz musician Miles Davis. It was released on August 17, 1959, by Columbia Records and is widely considered one of the greatest and most influential albums ever made.
+[4] THOUGHT: I keep getting the same general summary. Let me try current_info instead.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'Kind of Blue Miles Davis instruments track count'}
+[4] OBS: Real-time data for 'Kind of Blue Miles Davis instruments track count' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Miles Davis Kind of Blue tracklist saxophone piano bass'}
+[5] OBS: Page: Kind of Blue
+Summary: Kind of Blue is a studio album by American jazz musician Miles Davis. It was released on August 17, 1959, by Columbia Records and is widely considered one of the greatest and most influential albums ever made.
+FINAL: I don't have access to the detailed instrument and track listing information for Kind of Blue. Every search returned only a general summary without the specifics needed to answer the question.</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>46b63241,d9c46fce,9d91653a</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>SYN_L040_T3</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>TASK: Find out what instruments were used in the recording of Miles Davis's Kind of Blue and how many tracks the album contains.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Kind of Blue Miles Davis album instruments tracks'}
+[1] OBS: Page: Kind of Blue
+Summary: Kind of Blue is a studio album by American jazz musician Miles Davis. It was released on August 17, 1959, by Columbia Records and is widely considered one of the greatest and most influential albums ever made.
+[2] THOUGHT: The summary doesn't mention the instruments or track listing. Let me try a more specific search.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Kind of Blue album track listing musicians'}
+[2] OBS: Page: Kind of Blue
+Summary: Kind of Blue is a studio album by American jazz musician Miles Davis. It was released on August 17, 1959, by Columbia Records and is widely considered one of the greatest and most influential albums ever made.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Kind of Blue recording sessions personnel instruments'}
+[3] OBS: Page: Kind of Blue
+Summary: Kind of Blue is a studio album by American jazz musician Miles Davis. It was released on August 17, 1959, by Columbia Records and is widely considered one of the greatest and most influential albums ever made.</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>SYN_L040</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>SYN_L041</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>TASK: What was Frida Kahlo's artistic style and how many self-portraits did she paint in her lifetime?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Frida Kahlo artistic style self-portraits count'}
+[1] OBS: Page: Frida Kahlo
+Summary: Frida Kahlo de Rivera was a Mexican painter known for her many portraits, self-portraits, and works inspired by the nature and artifacts of Mexico. Her work has been celebrated in Mexico as emblematic of national and indigenous tradition and by feminists for its uncompromising depiction of the female experience and form.
+[2] THOUGHT: The summary mentions self-portraits but doesn't give a count or describe the style in detail. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Frida Kahlo number of self-portraits surrealism naive art'}
+[2] OBS: Page: Frida Kahlo
+Summary: Frida Kahlo de Rivera was a Mexican painter known for her many portraits, self-portraits, and works inspired by the nature and artifacts of Mexico. Her work has been celebrated in Mexico as emblematic of national and indigenous tradition and by feminists for its uncompromising depiction of the female experience and form.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Frida Kahlo paintings list style analysis'}
+[3] OBS: Page: Frida Kahlo
+Summary: Frida Kahlo de Rivera was a Mexican painter known for her many portraits, self-portraits, and works inspired by the nature and artifacts of Mexico. Her work has been celebrated in Mexico as emblematic of national and indigenous tradition and by feminists for its uncompromising depiction of the female experience and form.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'Frida Kahlo self-portraits total number artistic style'}
+[4] OBS: Real-time data for 'Frida Kahlo self-portraits total number artistic style' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I was unable to find the specific number of self-portraits Frida Kahlo painted or a detailed breakdown of her artistic style. The searches returned only a general summary each time.</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>46b63241,d9c46fce,9d91653a</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>SYN_L041_T3</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>TASK: What was Frida Kahlo's artistic style and how many self-portraits did she paint in her lifetime?
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Frida Kahlo artistic style self-portraits count'}
+[1] OBS: Page: Frida Kahlo
+Summary: Frida Kahlo de Rivera was a Mexican painter known for her many portraits, self-portraits, and works inspired by the nature and artifacts of Mexico. Her work has been celebrated in Mexico as emblematic of national and indigenous tradition and by feminists for its uncompromising depiction of the female experience and form.
+[2] THOUGHT: The summary mentions self-portraits but doesn't give a count or describe the style in detail. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Frida Kahlo number of self-portraits surrealism naive art'}
+[2] OBS: Page: Frida Kahlo
+Summary: Frida Kahlo de Rivera was a Mexican painter known for her many portraits, self-portraits, and works inspired by the nature and artifacts of Mexico. Her work has been celebrated in Mexico as emblematic of national and indigenous tradition and by feminists for its uncompromising depiction of the female experience and form.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Frida Kahlo paintings list style analysis'}
+[3] OBS: Page: Frida Kahlo
+Summary: Frida Kahlo de Rivera was a Mexican painter known for her many portraits, self-portraits, and works inspired by the nature and artifacts of Mexico. Her work has been celebrated in Mexico as emblematic of national and indigenous tradition and by feminists for its uncompromising depiction of the female experience and form.</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>SYN_L041</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>SYN_L042</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>TASK: Research the life of composer Johann Sebastian Bach and calculate how many years he lived.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Johann Sebastian Bach biography birth death'}
+[1] OBS: Page: Johann Sebastian Bach
+Summary: Johann Sebastian Bach was a German composer and musician of the late Baroque period. He is known for instrumental compositions such as the Brandenburg Concertos and the Goldberg Variations, and for vocal music such as the St Matthew Passion and the Mass in B minor.
+[2] THOUGHT: The summary doesn't include his birth and death years. I need those to calculate his lifespan. Let me search again.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Johann Sebastian Bach birth year death year lifespan'}
+[2] OBS: Page: Johann Sebastian Bach
+Summary: Johann Sebastian Bach was a German composer and musician of the late Baroque period. He is known for instrumental compositions such as the Brandenburg Concertos and the Goldberg Variations, and for vocal music such as the St Matthew Passion and the Mass in B minor.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Bach composer born 1685 died 1750'}
+[3] OBS: Page: Johann Sebastian Bach
+Summary: Johann Sebastian Bach was a German composer and musician of the late Baroque period. He is known for instrumental compositions such as the Brandenburg Concertos and the Goldberg Variations, and for vocal music such as the St Matthew Passion and the Mass in B minor.
+[4] THOUGHT: I keep receiving the same summary without the specific dates. Let me try current_info.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'Johann Sebastian Bach birth death dates'}
+[4] OBS: Real-time data for 'Johann Sebastian Bach birth death dates' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I was unable to retrieve the specific birth and death dates for Johann Sebastian Bach from the available tools, so I cannot calculate how many years he lived.</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>46b63241,d9c46fce,9d91653a</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>SYN_L042_T3</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>TASK: Research the life of composer Johann Sebastian Bach and calculate how many years he lived.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Johann Sebastian Bach biography birth death'}
+[1] OBS: Page: Johann Sebastian Bach
+Summary: Johann Sebastian Bach was a German composer and musician of the late Baroque period. He is known for instrumental compositions such as the Brandenburg Concertos and the Goldberg Variations, and for vocal music such as the St Matthew Passion and the Mass in B minor.
+[2] THOUGHT: The summary doesn't include his birth and death years. I need those to calculate his lifespan. Let me search again.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Johann Sebastian Bach birth year death year lifespan'}
+[2] OBS: Page: Johann Sebastian Bach
+Summary: Johann Sebastian Bach was a German composer and musician of the late Baroque period. He is known for instrumental compositions such as the Brandenburg Concertos and the Goldberg Variations, and for vocal music such as the St Matthew Passion and the Mass in B minor.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Bach composer born 1685 died 1750'}
+[3] OBS: Page: Johann Sebastian Bach
+Summary: Johann Sebastian Bach was a German composer and musician of the late Baroque period. He is known for instrumental compositions such as the Brandenburg Concertos and the Goldberg Variations, and for vocal music such as the St Matthew Passion and the Mass in B minor.</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>SYN_L042</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>SYN_L043</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>TASK: Find the names of the musicians who performed on The Beatles' Abbey Road album and how many songs are on it.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Abbey Road Beatles album musicians songs'}
+[1] OBS: Page: Abbey Road
+Summary: Abbey Road is the eleventh studio album by the English rock band the Beatles, released on 26 September 1969 by Apple Records. It is named after the London street where the Beatles' recording studio, Abbey Road Studios, is located.
+[2] THOUGHT: The summary gives general info but not the track count or full personnel list. Let me try a more targeted query.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Abbey Road album track listing personnel George Martin'}
+[2] OBS: Page: Abbey Road
+Summary: Abbey Road is the eleventh studio album by the English rock band the Beatles, released on 26 September 1969 by Apple Records. It is named after the London street where the Beatles' recording studio, Abbey Road Studios, is located.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Abbey Road 1969 full tracklist performers studio musicians'}
+[3] OBS: Page: Abbey Road
+Summary: Abbey Road is the eleventh studio album by the English rock band the Beatles, released on 26 September 1969 by Apple Records. It is named after the London street where the Beatles' recording studio, Abbey Road Studios, is located.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'Abbey Road Beatles performers track count'}
+[4] OBS: Real-time data for 'Abbey Road Beatles performers track count' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Abbey Road album songs list side one side two'}
+[5] OBS: Page: Abbey Road
+Summary: Abbey Road is the eleventh studio album by the English rock band the Beatles, released on 26 September 1969 by Apple Records. It is named after the London street where the Beatles' recording studio, Abbey Road Studios, is located.
+FINAL: I don't have access to the detailed track listing or full personnel information for Abbey Road. Each search returned only the same general album summary without the specifics I needed.</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>46b63241,d9c46fce,9d91653a</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>SYN_L043_T3</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>TASK: Find the names of the musicians who performed on The Beatles' Abbey Road album and how many songs are on it.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Abbey Road Beatles album musicians songs'}
+[1] OBS: Page: Abbey Road
+Summary: Abbey Road is the eleventh studio album by the English rock band the Beatles, released on 26 September 1969 by Apple Records. It is named after the London street where the Beatles' recording studio, Abbey Road Studios, is located.
+[2] THOUGHT: The summary gives general info but not the track count or full personnel list. Let me try a more targeted query.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Abbey Road album track listing personnel George Martin'}
+[2] OBS: Page: Abbey Road
+Summary: Abbey Road is the eleventh studio album by the English rock band the Beatles, released on 26 September 1969 by Apple Records. It is named after the London street where the Beatles' recording studio, Abbey Road Studios, is located.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Abbey Road 1969 full tracklist performers studio musicians'}
+[3] OBS: Page: Abbey Road
+Summary: Abbey Road is the eleventh studio album by the English rock band the Beatles, released on 26 September 1969 by Apple Records. It is named after the London street where the Beatles' recording studio, Abbey Road Studios, is located.</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>SYN_L043</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>SYN_L044</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 4]</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>TASK: What artistic techniques did Leonardo da Vinci use in painting the Mona Lisa?
+[1] THOUGHT: I'll look up the Mona Lisa to find information about the painting techniques Leonardo used.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Mona Lisa Leonardo da Vinci painting techniques'}
+[1] OBS: Page: Mona Lisa
+Summary: The Mona Lisa is a half-length portrait painting by Italian artist Leonardo da Vinci. Considered an archetypal masterpiece of the Italian Renaissance, it has been described as "the best known, the most visited, the most written about, the most sung about, the most parodied work of art in the world."
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Mona Lisa sfumato technique oil paint canvas method'}
+[2] OBS: Page: Mona Lisa
+Summary: The Mona Lisa is a half-length portrait painting by Italian artist Leonardo da Vinci. Considered an archetypal masterpiece of the Italian Renaissance, it has been described as "the best known, the most visited, the most written about, the most sung about, the most parodied work of art in the world."
+[3] THOUGHT: Still just getting a general description. Let me try searching for Leonardo da Vinci's techniques directly.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Leonardo da Vinci sfumato painting artistic methods Renaissance'}
+[3] OBS: Page: Leonardo da Vinci
+Summary: Leonardo di ser Piero da Vinci was an Italian polymath of the High Renaissance who was active as a painter, draughtsman, engineer, scientist, theorist, sculptor, and architect.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Mona Lisa analysis brushwork glazing artistic technique detail'}
+[4] OBS: Page: Mona Lisa
+Summary: The Mona Lisa is a half-length portrait painting by Italian artist Leonardo da Vinci. Considered an archetypal masterpiece of the Italian Renaissance, it has been described as "the best known, the most visited, the most written about, the most sung about, the most parodied work of art in the world."
+[5] ACTION: current_info
+[5] INPUT: {'query': 'Mona Lisa painting techniques sfumato Leonardo da Vinci'}
+[5] OBS: Real-time data for 'Mona Lisa painting techniques sfumato Leonardo da Vinci' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I was unable to retrieve detailed information about the specific artistic techniques Leonardo da Vinci used in painting the Mona Lisa. The tool searches only returned general summaries of the painting and its artist.</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>46b63241,d9c46fce,9d91653a</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>SYN_L044_T4</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 4]</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>TASK: What artistic techniques did Leonardo da Vinci use in painting the Mona Lisa?
+[1] THOUGHT: I'll look up the Mona Lisa to find information about the painting techniques Leonardo used.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Mona Lisa Leonardo da Vinci painting techniques'}
+[1] OBS: Page: Mona Lisa
+Summary: The Mona Lisa is a half-length portrait painting by Italian artist Leonardo da Vinci. Considered an archetypal masterpiece of the Italian Renaissance, it has been described as "the best known, the most visited, the most written about, the most sung about, the most parodied work of art in the world."
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Mona Lisa sfumato technique oil paint canvas method'}
+[2] OBS: Page: Mona Lisa
+Summary: The Mona Lisa is a half-length portrait painting by Italian artist Leonardo da Vinci. Considered an archetypal masterpiece of the Italian Renaissance, it has been described as "the best known, the most visited, the most written about, the most sung about, the most parodied work of art in the world."
+[3] THOUGHT: Still just getting a general description. Let me try searching for Leonardo da Vinci's techniques directly.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Leonardo da Vinci sfumato painting artistic methods Renaissance'}
+[3] OBS: Page: Leonardo da Vinci
+Summary: Leonardo di ser Piero da Vinci was an Italian polymath of the High Renaissance who was active as a painter, draughtsman, engineer, scientist, theorist, sculptor, and architect.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Mona Lisa analysis brushwork glazing artistic technique detail'}
+[4] OBS: Page: Mona Lisa
+Summary: The Mona Lisa is a half-length portrait painting by Italian artist Leonardo da Vinci. Considered an archetypal masterpiece of the Italian Renaissance, it has been described as "the best known, the most visited, the most written about, the most sung about, the most parodied work of art in the world."</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>SYN_L044</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>SYN_L045</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>TASK: Find the distance from Earth to the nearest star outside our solar system and the distance to the center of the Milky Way galaxy, then calculate the ratio between them.
+[1] THOUGHT: I'll start by looking up the distance to the nearest star outside our solar system.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'nearest star to Earth outside solar system distance'}
+[1] OBS: Page: Solar System
+Summary: The Solar System is the gravitationally bound system of the Sun and the objects that orbit it. It formed 4.6 billion years ago from the gravitational collapse of a giant molecular cloud. The vast majority of the system's mass is in the Sun, with most of the remaining mass contained in the planet Jupiter.
+[2] THOUGHT: That didn't return what I needed. Let me try a more specific query about Proxima Centauri.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'distance to nearest star Proxima Centauri light years'}
+[2] OBS: Page: Solar System
+Summary: The Solar System is the gravitationally bound system of the Sun and the objects that orbit it. It formed 4.6 billion years ago from the gravitational collapse of a giant molecular cloud. The vast majority of the system's mass is in the Sun, with most of the remaining mass contained in the planet Jupiter.
+[3] THOUGHT: Still getting the Solar System page. Let me try rephrasing the query.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Proxima Centauri nearest star distance parsecs'}
+[3] OBS: Page: Solar System
+Summary: The Solar System is the gravitationally bound system of the Sun and the objects that orbit it. It formed 4.6 billion years ago from the gravitational collapse of a giant molecular cloud. The vast majority of the system's mass is in the Sun, with most of the remaining mass contained in the planet Jupiter.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Alpha Centauri star system distance from Earth'}
+[4] OBS: Page: Solar System
+Summary: The Solar System is the gravitationally bound system of the Sun and the objects that orbit it. It formed 4.6 billion years ago from the gravitational collapse of a giant molecular cloud. The vast majority of the system's mass is in the Sun, with most of the remaining mass contained in the planet Jupiter.
+FINAL: I was unable to find the distance to the nearest star outside our solar system. The tool kept returning the Solar System page without the specific distance data I needed, so I cannot calculate the ratio between the two distances.</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>0efc9456,423d4398,17804dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>SYN_L045_T3</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>TASK: Find the distance from Earth to the nearest star outside our solar system and the distance to the center of the Milky Way galaxy, then calculate the ratio between them.
+[1] THOUGHT: I'll start by looking up the distance to the nearest star outside our solar system.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'nearest star to Earth outside solar system distance'}
+[1] OBS: Page: Solar System
+Summary: The Solar System is the gravitationally bound system of the Sun and the objects that orbit it. It formed 4.6 billion years ago from the gravitational collapse of a giant molecular cloud. The vast majority of the system's mass is in the Sun, with most of the remaining mass contained in the planet Jupiter.
+[2] THOUGHT: That didn't return what I needed. Let me try a more specific query about Proxima Centauri.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'distance to nearest star Proxima Centauri light years'}
+[2] OBS: Page: Solar System
+Summary: The Solar System is the gravitationally bound system of the Sun and the objects that orbit it. It formed 4.6 billion years ago from the gravitational collapse of a giant molecular cloud. The vast majority of the system's mass is in the Sun, with most of the remaining mass contained in the planet Jupiter.
+[3] THOUGHT: Still getting the Solar System page. Let me try rephrasing the query.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Proxima Centauri nearest star distance parsecs'}
+[3] OBS: Page: Solar System
+Summary: The Solar System is the gravitationally bound system of the Sun and the objects that orbit it. It formed 4.6 billion years ago from the gravitational collapse of a giant molecular cloud. The vast majority of the system's mass is in the Sun, with most of the remaining mass contained in the planet Jupiter.</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>SYN_L045</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>SYN_L046</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 5]</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>TASK: What is the surface temperature of Venus and the surface temperature of Mars? Calculate how many times hotter Venus is than Mars.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Venus surface temperature'}
+[1] OBS: Page: Venus
+Summary: Venus is the second planet from the Sun. It is a terrestrial planet and is the closest in mass and size to its orbital neighbour Earth. Venus has by far the densest atmosphere of the terrestrial planets, composed mostly of carbon dioxide with a thick, global sulfuric acid cloud cover. The planet is named after and associated with the Roman goddess of love and beauty.
+[2] THOUGHT: The summary didn't include the specific temperature. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Venus average surface temperature degrees Celsius'}
+[2] OBS: Page: Venus
+Summary: Venus is the second planet from the Sun. It is a terrestrial planet and is the closest in mass and size to its orbital neighbour Earth. Venus has by far the densest atmosphere of the terrestrial planets, composed mostly of carbon dioxide with a thick, global sulfuric acid cloud cover. The planet is named after and associated with the Roman goddess of love and beauty.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Mars surface temperature average'}
+[3] OBS: Page: Mars
+Summary: Mars is the fourth planet from the Sun. The surface of Mars is orange-red because it is covered in iron(II) oxide dust, giving it the nickname "the Red Planet". Mars is among the brightest objects in Earth's sky and its high-contrast albedo features have driven interest from astronomers.
+[4] THOUGHT: Neither result gave me specific temperatures. Let me try querying for Mars temperature more precisely.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Mars average surface temperature Celsius Kelvin'}
+[4] OBS: Page: Mars
+Summary: Mars is the fourth planet from the Sun. The surface of Mars is orange-red because it is covered in iron(II) oxide dust, giving it the nickname "the Red Planet". Mars is among the brightest objects in Earth's sky and its high-contrast albedo features have driven interest from astronomers.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Venus temperature hottest planet surface'}
+[5] OBS: Page: Venus
+Summary: Venus is the second planet from the Sun. It is a terrestrial planet and is the closest in mass and size to its orbital neighbour Earth. Venus has by far the densest atmosphere of the terrestrial planets, composed mostly of carbon dioxide with a thick, global sulfuric acid cloud cover. The planet is named after and associated with the Roman goddess of love and beauty.
+FINAL: I was unable to retrieve the specific surface temperatures of Venus or Mars from the available tool. The Wikipedia summaries returned only general descriptions without the numerical temperature values I needed to perform the calculation.</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>0efc9456,423d4398,17804dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>SYN_L046_T5</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 5]</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>TASK: What is the surface temperature of Venus and the surface temperature of Mars? Calculate how many times hotter Venus is than Mars.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Venus surface temperature'}
+[1] OBS: Page: Venus
+Summary: Venus is the second planet from the Sun. It is a terrestrial planet and is the closest in mass and size to its orbital neighbour Earth. Venus has by far the densest atmosphere of the terrestrial planets, composed mostly of carbon dioxide with a thick, global sulfuric acid cloud cover. The planet is named after and associated with the Roman goddess of love and beauty.
+[2] THOUGHT: The summary didn't include the specific temperature. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Venus average surface temperature degrees Celsius'}
+[2] OBS: Page: Venus
+Summary: Venus is the second planet from the Sun. It is a terrestrial planet and is the closest in mass and size to its orbital neighbour Earth. Venus has by far the densest atmosphere of the terrestrial planets, composed mostly of carbon dioxide with a thick, global sulfuric acid cloud cover. The planet is named after and associated with the Roman goddess of love and beauty.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Mars surface temperature average'}
+[3] OBS: Page: Mars
+Summary: Mars is the fourth planet from the Sun. The surface of Mars is orange-red because it is covered in iron(II) oxide dust, giving it the nickname "the Red Planet". Mars is among the brightest objects in Earth's sky and its high-contrast albedo features have driven interest from astronomers.
+[4] THOUGHT: Neither result gave me specific temperatures. Let me try querying for Mars temperature more precisely.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Mars average surface temperature Celsius Kelvin'}
+[4] OBS: Page: Mars
+Summary: Mars is the fourth planet from the Sun. The surface of Mars is orange-red because it is covered in iron(II) oxide dust, giving it the nickname "the Red Planet". Mars is among the brightest objects in Earth's sky and its high-contrast albedo features have driven interest from astronomers.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Venus temperature hottest planet surface'}
+[5] OBS: Page: Venus
+Summary: Venus is the second planet from the Sun. It is a terrestrial planet and is the closest in mass and size to its orbital neighbour Earth. Venus has by far the densest atmosphere of the terrestrial planets, composed mostly of carbon dioxide with a thick, global sulfuric acid cloud cover. The planet is named after and associated with the Roman goddess of love and beauty.</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>SYN_L046</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>SYN_L047</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>TASK: Find the orbital period of Jupiter and the orbital period of Saturn, then calculate how much longer Saturn's year is compared to Jupiter's.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Jupiter orbital period years'}
+[1] OBS: Page: Jupiter
+Summary: Jupiter is the fifth planet from the Sun and the largest in the Solar System. It is a gas giant with a mass more than 2.5 times that of all the other planets in the Solar System combined, and slightly less than one-thousandth the mass of the Sun. Jupiter is the third brightest natural object in the night sky after the Moon and Venus, and has been observed since prehistoric times.
+[2] THOUGHT: The summary doesn't mention the orbital period specifically. Let me try Saturn next and then try more specific queries.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Saturn orbital period revolution around Sun'}
+[2] OBS: Page: Saturn
+Summary: Saturn is the sixth planet from the Sun and the second largest in the Solar System, after Jupiter. It is a gas giant with an average radius of about nine and a half times that of Earth. It has only one-eighth the average density of Earth, but is over 95 times more massive.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Jupiter year length Earth years orbital revolution'}
+[3] OBS: Page: Jupiter
+Summary: Jupiter is the fifth planet from the Sun and the largest in the Solar System. It is a gas giant with a mass more than 2.5 times that of all the other planets in the Solar System combined, and slightly less than one-thousandth the mass of the Sun. Jupiter is the third brightest natural object in the night sky after the Moon and Venus, and has been observed since prehistoric times.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Saturn year length orbital period Earth years'}
+[4] OBS: Page: Saturn
+Summary: Saturn is the sixth planet from the Sun and the second largest in the Solar System, after Jupiter. It is a gas giant with an average radius of about nine and a half times that of Earth. It has only one-eighth the average density of Earth, but is over 95 times more massive.
+[5] THOUGHT: I keep getting general summaries. Let me try using current_info to see if I can get more specific data.
+[5] ACTION: current_info
+[5] INPUT: {'query': 'Jupiter orbital period in Earth years'}
+[5] OBS: No current information available for this query.
+[6] ACTION: current_info
+[6] INPUT: {'query': 'Saturn orbital period in Earth years'}
+[6] OBS: No current information available for this query.
+FINAL: I was unable to find the specific orbital periods for Jupiter and Saturn. Both the Wikipedia summaries and current_info tool failed to return the numerical data needed to calculate the difference between Saturn's and Jupiter's orbital periods.</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>0efc9456,423d4398,17804dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>SYN_L047_T3</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>TASK: Find the orbital period of Jupiter and the orbital period of Saturn, then calculate how much longer Saturn's year is compared to Jupiter's.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Jupiter orbital period years'}
+[1] OBS: Page: Jupiter
+Summary: Jupiter is the fifth planet from the Sun and the largest in the Solar System. It is a gas giant with a mass more than 2.5 times that of all the other planets in the Solar System combined, and slightly less than one-thousandth the mass of the Sun. Jupiter is the third brightest natural object in the night sky after the Moon and Venus, and has been observed since prehistoric times.
+[2] THOUGHT: The summary doesn't mention the orbital period specifically. Let me try Saturn next and then try more specific queries.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Saturn orbital period revolution around Sun'}
+[2] OBS: Page: Saturn
+Summary: Saturn is the sixth planet from the Sun and the second largest in the Solar System, after Jupiter. It is a gas giant with an average radius of about nine and a half times that of Earth. It has only one-eighth the average density of Earth, but is over 95 times more massive.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Jupiter year length Earth years orbital revolution'}
+[3] OBS: Page: Jupiter
+Summary: Jupiter is the fifth planet from the Sun and the largest in the Solar System. It is a gas giant with a mass more than 2.5 times that of all the other planets in the Solar System combined, and slightly less than one-thousandth the mass of the Sun. Jupiter is the third brightest natural object in the night sky after the Moon and Venus, and has been observed since prehistoric times.</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>SYN_L047</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>SYN_L048</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>TASK: Look up the diameter of the Andromeda Galaxy and the diameter of the Milky Way and find the percentage difference between them.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Andromeda Galaxy diameter size light years'}
+[1] OBS: Page: Andromeda Galaxy
+Summary: The Andromeda Galaxy, also known as Messier 31, is a barred spiral galaxy and is the nearest major galaxy to the Milky Way. It was named after the princess Andromeda in Greek mythology. Andromeda is the largest galaxy of the Local Group, which also contains the Milky Way, the Triangulum Galaxy, and about 54 other smaller galaxies.
+[2] THOUGHT: The summary says Andromeda is the largest in the Local Group but doesn't give a specific diameter. Let me search for the Milky Way diameter.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Milky Way galaxy diameter kiloparsecs light years'}
+[2] OBS: Page: Milky Way
+Summary: The Milky Way is the galaxy that contains the Solar System, with the latter being located within the Outer Arm of the galaxy. Earth and the Solar System are situated within the disc of the Milky Way, at a distance of 26,660 light-years from the Galactic Center.
+[3] THOUGHT: Still no specific diameter figures. Let me try more targeted searches.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Andromeda Galaxy size diameter kilometers parsecs'}
+[3] OBS: Page: Andromeda Galaxy
+Summary: The Andromeda Galaxy, also known as Messier 31, is a barred spiral galaxy and is the nearest major galaxy to the Milky Way. It was named after the princess Andromeda in Greek mythology. Andromeda is the largest galaxy of the Local Group, which also contains the Milky Way, the Triangulum Galaxy, and about 54 other smaller galaxies.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Milky Way size diameter across light years measurement'}
+[4] OBS: Page: Milky Way
+Summary: The Milky Way is the galaxy that contains the Solar System, with the latter being located within the Outer Arm of the galaxy. Earth and the Solar System are situated within the disc of the Milky Way, at a distance of 26,660 light-years from the Galactic Center.
+FINAL: I was unable to retrieve the specific diameter values for either the Andromeda Galaxy or the Milky Way. The Wikipedia summaries returned general descriptions without the numerical measurements needed to calculate a percentage difference.</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>0efc9456,423d4398,17804dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>SYN_L048_T3</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>TASK: Look up the diameter of the Andromeda Galaxy and the diameter of the Milky Way and find the percentage difference between them.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Andromeda Galaxy diameter size light years'}
+[1] OBS: Page: Andromeda Galaxy
+Summary: The Andromeda Galaxy, also known as Messier 31, is a barred spiral galaxy and is the nearest major galaxy to the Milky Way. It was named after the princess Andromeda in Greek mythology. Andromeda is the largest galaxy of the Local Group, which also contains the Milky Way, the Triangulum Galaxy, and about 54 other smaller galaxies.
+[2] THOUGHT: The summary says Andromeda is the largest in the Local Group but doesn't give a specific diameter. Let me search for the Milky Way diameter.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Milky Way galaxy diameter kiloparsecs light years'}
+[2] OBS: Page: Milky Way
+Summary: The Milky Way is the galaxy that contains the Solar System, with the latter being located within the Outer Arm of the galaxy. Earth and the Solar System are situated within the disc of the Milky Way, at a distance of 26,660 light-years from the Galactic Center.
+[3] THOUGHT: Still no specific diameter figures. Let me try more targeted searches.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Andromeda Galaxy size diameter kilometers parsecs'}
+[3] OBS: Page: Andromeda Galaxy
+Summary: The Andromeda Galaxy, also known as Messier 31, is a barred spiral galaxy and is the nearest major galaxy to the Milky Way. It was named after the princess Andromeda in Greek mythology. Andromeda is the largest galaxy of the Local Group, which also contains the Milky Way, the Triangulum Galaxy, and about 54 other smaller galaxies.</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>SYN_L048</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>SYN_L049</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>TASK: What is the mass of the Sun compared to the mass of the Earth? Find both values and compute the ratio.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'mass of the Sun kilograms'}
+[1] OBS: Page: Sun
+Summary: The Sun is the star at the center of the Solar System. It is a massive, nearly perfect sphere of hot plasma, heated to incandescence by nuclear fusion reactions in its core. The Sun radiates this energy mainly as light, ultraviolet, and infrared radiation, and is the most important source of energy for life on Earth.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'mass of Earth kilograms'}
+[2] OBS: Page: Earth
+Summary: Earth is the third planet from the Sun and the only astronomical object known to harbor life. This is enabled by Earth being an ocean world, the only one in the Solar System sustaining liquid surface water. Almost all of Earth's water is contained in its global ocean, covering 70.8% of Earth's crust.
+[3] THOUGHT: Neither summary gave me the actual mass values. Let me try more targeted queries.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'solar mass Sun total mass value'}
+[3] OBS: Page: Sun
+Summary: The Sun is the star at the center of the Solar System. It is a massive, nearly perfect sphere of hot plasma, heated to incandescence by nuclear fusion reactions in its core. The Sun radiates this energy mainly as light, ultraviolet, and infrared radiation, and is the most important source of energy for life on Earth.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Earth mass value scientific notation'}
+[4] OBS: Page: Earth
+Summary: Earth is the third planet from the Sun and the only astronomical object known to harbor life. This is enabled by Earth being an ocean world, the only one in the Solar System sustaining liquid surface water. Almost all of Earth's water is contained in its global ocean, covering 70.8% of Earth's crust.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Sun mass compared to Earth times heavier'}
+[5] OBS: Page: Sun
+Summary: The Sun is the star at the center of the Solar System. It is a massive, nearly perfect sphere of hot plasma, heated to incandescence by nuclear fusion reactions in its core. The Sun radiates this energy mainly as light, ultraviolet, and infrared radiation, and is the most important source of energy for life on Earth.
+FINAL: I don't have access to the specific mass values for the Sun and Earth. Each query returned only general summary paragraphs without numerical data, making it impossible to compute the ratio between them.</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>0efc9456,423d4398,17804dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>SYN_L049_T5</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>TASK: What is the mass of the Sun compared to the mass of the Earth? Find both values and compute the ratio.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'mass of the Sun kilograms'}
+[1] OBS: Page: Sun
+Summary: The Sun is the star at the center of the Solar System. It is a massive, nearly perfect sphere of hot plasma, heated to incandescence by nuclear fusion reactions in its core. The Sun radiates this energy mainly as light, ultraviolet, and infrared radiation, and is the most important source of energy for life on Earth.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'mass of Earth kilograms'}
+[2] OBS: Page: Earth
+Summary: Earth is the third planet from the Sun and the only astronomical object known to harbor life. This is enabled by Earth being an ocean world, the only one in the Solar System sustaining liquid surface water. Almost all of Earth's water is contained in its global ocean, covering 70.8% of Earth's crust.
+[3] THOUGHT: Neither summary gave me the actual mass values. Let me try more targeted queries.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'solar mass Sun total mass value'}
+[3] OBS: Page: Sun
+Summary: The Sun is the star at the center of the Solar System. It is a massive, nearly perfect sphere of hot plasma, heated to incandescence by nuclear fusion reactions in its core. The Sun radiates this energy mainly as light, ultraviolet, and infrared radiation, and is the most important source of energy for life on Earth.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Earth mass value scientific notation'}
+[4] OBS: Page: Earth
+Summary: Earth is the third planet from the Sun and the only astronomical object known to harbor life. This is enabled by Earth being an ocean world, the only one in the Solar System sustaining liquid surface water. Almost all of Earth's water is contained in its global ocean, covering 70.8% of Earth's crust.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Sun mass compared to Earth times heavier'}
+[5] OBS: Page: Sun
+Summary: The Sun is the star at the center of the Solar System. It is a massive, nearly perfect sphere of hot plasma, heated to incandescence by nuclear fusion reactions in its core. The Sun radiates this energy mainly as light, ultraviolet, and infrared radiation, and is the most important source of energy for life on Earth.</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>SYN_L049</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>SYN_L050</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>TASK: Find how long it takes light to travel from the Sun to Neptune and from the Sun to Pluto, and calculate the difference in travel time.
+[1] THOUGHT: I'll look up the distance from the Sun to Neptune first, then to Pluto, and use the speed of light to compute travel times.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Neptune distance from Sun astronomical units light minutes'}
+[1] OBS: Page: Neptune
+Summary: Neptune is the eighth and farthest known planet from the Sun. It is the fourth-largest planet in the Solar System by diameter, the third-most-massive planet, and the densest giant planet. It is 17 times the mass of Earth.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Pluto distance from Sun light minutes AU'}
+[2] OBS: Page: Pluto
+Summary: Pluto is a dwarf planet in the Kuiper Belt, a ring of bodies beyond the orbit of Neptune. It was the first object discovered in the Kuiper Belt and remains the largest known body in that area. Pluto was discovered by Clive Tombaugh in 1930.
+[3] THOUGHT: Neither returned specific distance figures. Let me search more specifically.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Neptune average distance Sun kilometers AU value'}
+[3] OBS: Page: Neptune
+Summary: Neptune is the eighth and farthest known planet from the Sun. It is the fourth-largest planet in the Solar System by diameter, the third-most-massive planet, and the densest giant planet. It is 17 times the mass of Earth.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Pluto average distance from Sun kilometers astronomical units'}
+[4] OBS: Page: Pluto
+Summary: Pluto is a dwarf planet in the Kuiper Belt, a ring of bodies beyond the orbit of Neptune. It was the first object discovered in the Kuiper Belt and remains the largest known body in that area. Pluto was discovered by Clive Tombaugh in 1930.
+[5] ACTION: current_info
+[5] INPUT: {'query': 'Neptune distance from Sun in light minutes'}
+[5] OBS: No current information available for this query.
+FINAL: I was unable to find the specific distances from the Sun to Neptune and Pluto. Without those values, I cannot calculate the light travel times or the difference between them.</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>0efc9456,423d4398,17804dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>SYN_L050_T3</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>TASK: Find how long it takes light to travel from the Sun to Neptune and from the Sun to Pluto, and calculate the difference in travel time.
+[1] THOUGHT: I'll look up the distance from the Sun to Neptune first, then to Pluto, and use the speed of light to compute travel times.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Neptune distance from Sun astronomical units light minutes'}
+[1] OBS: Page: Neptune
+Summary: Neptune is the eighth and farthest known planet from the Sun. It is the fourth-largest planet in the Solar System by diameter, the third-most-massive planet, and the densest giant planet. It is 17 times the mass of Earth.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Pluto distance from Sun light minutes AU'}
+[2] OBS: Page: Pluto
+Summary: Pluto is a dwarf planet in the Kuiper Belt, a ring of bodies beyond the orbit of Neptune. It was the first object discovered in the Kuiper Belt and remains the largest known body in that area. Pluto was discovered by Clive Tombaugh in 1930.
+[3] THOUGHT: Neither returned specific distance figures. Let me search more specifically.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Neptune average distance Sun kilometers AU value'}
+[3] OBS: Page: Neptune
+Summary: Neptune is the eighth and farthest known planet from the Sun. It is the fourth-largest planet in the Solar System by diameter, the third-most-massive planet, and the densest giant planet. It is 17 times the mass of Earth.</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>SYN_L050</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>SYN_L051</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>TASK: Find the magnitude of the largest earthquake ever recorded and where it occurred.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'largest earthquake ever recorded magnitude'}
+[1] OBS: Page: Lists of earthquakes
+Summary: This article lists notable earthquakes that have been recorded historically. Earthquakes are measured using seismometers and the magnitude is calculated using various scales including the Richter scale and moment magnitude scale. The list includes earthquakes that caused significant damage or casualties throughout history.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'most powerful earthquake in history magnitude location'}
+[2] OBS: Page: Lists of earthquakes
+Summary: This article lists notable earthquakes that have been recorded historically. Earthquakes are measured using seismometers and the magnitude is calculated using various scales including the Richter scale and moment magnitude scale. The list includes earthquakes that caused significant damage or casualties throughout history.
+[3] THOUGHT: I need to find the specific magnitude and location of the largest earthquake ever recorded. Let me try a more specific search.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'strongest earthquake recorded history location magnitude scale'}
+[3] OBS: Page: Lists of earthquakes
+Summary: This article lists notable earthquakes that have been recorded historically. Earthquakes are measured using seismometers and the magnitude is calculated using various scales including the Richter scale and moment magnitude scale. The list includes earthquakes that caused significant damage or casualties throughout history.
+FINAL: I was unable to find the specific magnitude and location of the largest earthquake ever recorded. The search results kept returning only a general overview page without the specific details needed.</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>0b3f5839,b37fb3ed,8ddf9faa</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>SYN_L051_T3</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>TASK: Find the magnitude of the largest earthquake ever recorded and where it occurred.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'largest earthquake ever recorded magnitude'}
+[1] OBS: Page: Lists of earthquakes
+Summary: This article lists notable earthquakes that have been recorded historically. Earthquakes are measured using seismometers and the magnitude is calculated using various scales including the Richter scale and moment magnitude scale. The list includes earthquakes that caused significant damage or casualties throughout history.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'most powerful earthquake in history magnitude location'}
+[2] OBS: Page: Lists of earthquakes
+Summary: This article lists notable earthquakes that have been recorded historically. Earthquakes are measured using seismometers and the magnitude is calculated using various scales including the Richter scale and moment magnitude scale. The list includes earthquakes that caused significant damage or casualties throughout history.
+[3] THOUGHT: I need to find the specific magnitude and location of the largest earthquake ever recorded. Let me try a more specific search.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'strongest earthquake recorded history location magnitude scale'}
+[3] OBS: Page: Lists of earthquakes
+Summary: This article lists notable earthquakes that have been recorded historically. Earthquakes are measured using seismometers and the magnitude is calculated using various scales including the Richter scale and moment magnitude scale. The list includes earthquakes that caused significant damage or casualties throughout history.</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>SYN_L051</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>SYN_L052</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>TASK: Find the depth of the Mariana Trench and the depth of the Tonga Trench and determine which is deeper and by how many meters.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Mariana Trench depth meters'}
+[1] OBS: Page: Mariana Trench
+Summary: The Mariana Trench is an oceanic trench located in the western Pacific Ocean, east of the Mariana Islands. It is the deepest oceanic trench on Earth. The trench is roughly crescent-shaped and measures about 2,550 km in length and 69 km in width.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Tonga Trench depth meters'}
+[2] OBS: Page: Tonga Trench
+Summary: The Tonga Trench is an oceanic trench located in the south Pacific Ocean. It is the second deepest trench in the world and the deepest in the Southern Hemisphere. The trench is located northeast of New Zealand and north of Tonga.
+[3] THOUGHT: I got general information about both trenches but no specific depth values. Let me search more specifically for the depth measurements.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Mariana Trench maximum depth exact measurement'}
+[3] OBS: Page: Mariana Trench
+Summary: The Mariana Trench is an oceanic trench located in the western Pacific Ocean, east of the Mariana Islands. It is the deepest oceanic trench on Earth. The trench is roughly crescent-shaped and measures about 2,550 km in length and 69 km in width.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'Tonga Trench maximum depth exact measurement kilometers'}
+[4] OBS: Page: Tonga Trench
+Summary: The Tonga Trench is an oceanic trench located in the south Pacific Ocean. It is the second deepest trench in the world and the deepest in the Southern Hemisphere. The trench is located northeast of New Zealand and north of Tonga.
+[5] THOUGHT: I still don't have the specific depth figures. Let me try using current_info to get these measurements.
+[5] ACTION: current_info
+[5] INPUT: {'query': 'Mariana Trench depth in meters'}
+[5] OBS: Real-time data for 'Mariana Trench depth in meters' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[6] ACTION: current_info
+[6] INPUT: {'query': 'Tonga Trench depth in meters'}
+[6] OBS: Real-time data for 'Tonga Trench depth in meters' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I don't have access to the specific depth measurements for the Mariana Trench and the Tonga Trench. I was unable to retrieve the numerical depth values needed to compare the two trenches.</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>0b3f5839,b37fb3ed,8ddf9faa</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>SYN_L052_T3</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>TASK: Find the depth of the Mariana Trench and the depth of the Tonga Trench and determine which is deeper and by how many meters.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Mariana Trench depth meters'}
+[1] OBS: Page: Mariana Trench
+Summary: The Mariana Trench is an oceanic trench located in the western Pacific Ocean, east of the Mariana Islands. It is the deepest oceanic trench on Earth. The trench is roughly crescent-shaped and measures about 2,550 km in length and 69 km in width.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Tonga Trench depth meters'}
+[2] OBS: Page: Tonga Trench
+Summary: The Tonga Trench is an oceanic trench located in the south Pacific Ocean. It is the second deepest trench in the world and the deepest in the Southern Hemisphere. The trench is located northeast of New Zealand and north of Tonga.
+[3] THOUGHT: I got general information about both trenches but no specific depth values. Let me search more specifically for the depth measurements.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Mariana Trench maximum depth exact measurement'}
+[3] OBS: Page: Mariana Trench
+Summary: The Mariana Trench is an oceanic trench located in the western Pacific Ocean, east of the Mariana Islands. It is the deepest oceanic trench on Earth. The trench is roughly crescent-shaped and measures about 2,550 km in length and 69 km in width.</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>SYN_L052</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>SYN_L053</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>TASK: Find how many people were killed in the 1980 Mount St. Helens eruption and how much ash was produced.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Mount St. Helens eruption 1980 deaths ash'}
+[1] OBS: Page: Mount St. Helens
+Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.
+[2] THOUGHT: I got general information about Mount St. Helens but not the specific death toll and ash production from the 1980 eruption. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': '1980 Mount St. Helens eruption casualties fatalities'}
+[2] OBS: Page: Mount St. Helens
+Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': '1980 eruption Mount St Helens death toll volcanic ash volume'}
+[3] OBS: Page: Mount St. Helens
+Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'May 18 1980 volcanic eruption Washington state people killed'}
+[4] OBS: Page: Mount St. Helens
+Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.
+FINAL: I was unable to find the specific death toll and ash production figures for the 1980 Mount St. Helens eruption. All my searches returned only general information about the volcano without the specific statistics I needed.</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>0b3f5839,b37fb3ed,8ddf9faa</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>SYN_L053_T4</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>TASK: Find how many people were killed in the 1980 Mount St. Helens eruption and how much ash was produced.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Mount St. Helens eruption 1980 deaths ash'}
+[1] OBS: Page: Mount St. Helens
+Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.
+[2] THOUGHT: I got general information about Mount St. Helens but not the specific death toll and ash production from the 1980 eruption. Let me search more specifically.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': '1980 Mount St. Helens eruption casualties fatalities'}
+[2] OBS: Page: Mount St. Helens
+Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': '1980 eruption Mount St Helens death toll volcanic ash volume'}
+[3] OBS: Page: Mount St. Helens
+Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.
+[4] ACTION: wikipedia_lookup
+[4] INPUT: {'query': 'May 18 1980 volcanic eruption Washington state people killed'}
+[4] OBS: Page: Mount St. Helens
+Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>SYN_L053</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>SYN_L054</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>TASK: Find the date and location of the 2004 Indian Ocean tsunami and how many countries were affected.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': '2004 Indian Ocean tsunami date location countries affected'}
+[1] OBS: Page: Indian Ocean
+Summary: The Indian Ocean is the third-largest of the world's five oceanic divisions, covering an area of 70,560,000 km2. It is bounded by Asia to the north, Africa to the west, and Australia to the east. To the south it is bounded by the Southern Ocean or Antarctica, depending on the definition used.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': '2004 tsunami Indonesia earthquake countries death toll'}
+[2] OBS: Page: Indian Ocean
+Summary: The Indian Ocean is the third-largest of the world's five oceanic divisions, covering an area of 70,560,000 km2. It is bounded by Asia to the north, Africa to the west, and Australia to the east. To the south it is bounded by the Southern Ocean or Antarctica, depending on the definition used.
+[3] THOUGHT: My searches are returning the wrong page. Let me try a different query to find the specific tsunami event.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': '2004 Boxing Day tsunami earthquake Sumatra affected nations'}
+[3] OBS: Page: Indian Ocean
+Summary: The Indian Ocean is the third-largest of the world's five oceanic divisions, covering an area of 70,560,000 km2. It is bounded by Asia to the north, Africa to the west, and Australia to the east. To the south it is bounded by the Southern Ocean or Antarctica, depending on the definition used.
+[4] ACTION: current_info
+[4] INPUT: {'query': '2004 Indian Ocean tsunami countries affected'}
+[4] OBS: Real-time data for '2004 Indian Ocean tsunami countries affected' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I was unable to find the specific details about the 2004 Indian Ocean tsunami, including the number of countries affected. My searches repeatedly returned general information about the Indian Ocean rather than the tsunami event itself.</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>0b3f5839,b37fb3ed,8ddf9faa</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>SYN_L054_T3</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>TASK: Find the date and location of the 2004 Indian Ocean tsunami and how many countries were affected.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': '2004 Indian Ocean tsunami date location countries affected'}
+[1] OBS: Page: Indian Ocean
+Summary: The Indian Ocean is the third-largest of the world's five oceanic divisions, covering an area of 70,560,000 km2. It is bounded by Asia to the north, Africa to the west, and Australia to the east. To the south it is bounded by the Southern Ocean or Antarctica, depending on the definition used.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': '2004 tsunami Indonesia earthquake countries death toll'}
+[2] OBS: Page: Indian Ocean
+Summary: The Indian Ocean is the third-largest of the world's five oceanic divisions, covering an area of 70,560,000 km2. It is bounded by Asia to the north, Africa to the west, and Australia to the east. To the south it is bounded by the Southern Ocean or Antarctica, depending on the definition used.
+[3] THOUGHT: My searches are returning the wrong page. Let me try a different query to find the specific tsunami event.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': '2004 Boxing Day tsunami earthquake Sumatra affected nations'}
+[3] OBS: Page: Indian Ocean
+Summary: The Indian Ocean is the third-largest of the world's five oceanic divisions, covering an area of 70,560,000 km2. It is bounded by Asia to the north, Africa to the west, and Australia to the east. To the south it is bounded by the Southern Ocean or Antarctica, depending on the definition used.</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>SYN_L054</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>SYN_L055</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>TASK: Find the flow rate of lava during the 2018 Kilauea eruption in Hawaii and how many homes were destroyed.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': '2018 Kilauea eruption Hawaii lava flow rate homes destroyed'}
+[1] OBS: Page: Kīlauea
+Summary: Kīlauea is a currently active shield volcano in the Hawaiian Islands, and the most active of the five volcanoes that together form the island of Hawaiʻi. Located along the southeastern shore of the island, the volcano is between 210,000 and 280,000 years old.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': '2018 lower East Rift Zone eruption Kilauea structures destroyed lava rate'}
+[2] OBS: Page: Kīlauea
+Summary: Kīlauea is a currently active shield volcano in the Hawaiian Islands, and the most active of the five volcanoes that together form the island of Hawaiʻi. Located along the southeastern shore of the island, the volcano is between 210,000 and 280,000 years old.
+[3] THOUGHT: The search keeps returning the general Kilauea page rather than the 2018 eruption specifically. Let me try to search directly for the 2018 eruption event.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Kilauea 2018 volcanic eruption damage statistics'}
+[3] OBS: Page: Kīlauea
+Summary: Kīlauea is a currently active shield volcano in the Hawaiian Islands, and the most active of the five volcanoes that together form the island of Hawaiʻi. Located along the southeastern shore of the island, the volcano is between 210,000 and 280,000 years old.
+[4] THOUGHT: I'm still not getting specific information about the 2018 eruption. Let me try current_info.
+[4] ACTION: current_info
+[4] INPUT: {'query': '2018 Kilauea eruption homes destroyed lava flow rate'}
+[4] OBS: Real-time data for '2018 Kilauea eruption homes destroyed lava flow rate' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+[5] ACTION: wikipedia_lookup
+[5] INPUT: {'query': 'Hawaii volcanic eruption 2018 houses destroyed number'}
+[5] OBS: Page: Kīlauea
+Summary: Kīlauea is a currently active shield volcano in the Hawaiian Islands, and the most active of the five volcanoes that together form the island of Hawaiʻi. Located along the southeastern shore of the island, the volcano is between 210,000 and 280,000 years old.
+FINAL: I don't have access to the specific statistics for the 2018 Kilauea eruption. My repeated searches only returned general information about the Kilauea volcano and I was unable to find the lava flow rate or the number of homes destroyed.</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>0b3f5839,b37fb3ed,8ddf9faa</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>SYN_L055_T3</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>TASK: Find the flow rate of lava during the 2018 Kilauea eruption in Hawaii and how many homes were destroyed.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': '2018 Kilauea eruption Hawaii lava flow rate homes destroyed'}
+[1] OBS: Page: Kīlauea
+Summary: Kīlauea is a currently active shield volcano in the Hawaiian Islands, and the most active of the five volcanoes that together form the island of Hawaiʻi. Located along the southeastern shore of the island, the volcano is between 210,000 and 280,000 years old.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': '2018 lower East Rift Zone eruption Kilauea structures destroyed lava rate'}
+[2] OBS: Page: Kīlauea
+Summary: Kīlauea is a currently active shield volcano in the Hawaiian Islands, and the most active of the five volcanoes that together form the island of Hawaiʻi. Located along the southeastern shore of the island, the volcano is between 210,000 and 280,000 years old.
+[3] THOUGHT: The search keeps returning the general Kilauea page rather than the 2018 eruption specifically. Let me try to search directly for the 2018 eruption event.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Kilauea 2018 volcanic eruption damage statistics'}
+[3] OBS: Page: Kīlauea
+Summary: Kīlauea is a currently active shield volcano in the Hawaiian Islands, and the most active of the five volcanoes that together form the island of Hawaiʻi. Located along the southeastern shore of the island, the volcano is between 210,000 and 280,000 years old.</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>SYN_L055</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>SYN_L056</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>TASK: Find the total area of land lost to erosion along the Louisiana coastline each year and calculate how much would be lost in 50 years at that rate.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Louisiana coastal erosion land loss per year acres'}
+[1] OBS: Page: Louisiana
+Summary: Louisiana is a state in the Deep South and South Central regions of the United States. It is the 19th-smallest by area and the 25th most-populous of the 50 U.S. states. Its capital is Baton Rouge, and its largest city is New Orleans.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Louisiana coast land erosion rate square miles annually'}
+[2] OBS: Page: Louisiana
+Summary: Louisiana is a state in the Deep South and South Central regions of the United States. It is the 19th-smallest by area and the 25th most-populous of the 50 U.S. states. Its capital is Baton Rouge, and its largest city is New Orleans.
+[3] THOUGHT: I need more specific information about the coastal erosion rate. Let me try a more targeted search.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Louisiana wetlands coastal erosion land loss rate statistics'}
+[3] OBS: Page: Louisiana
+Summary: Louisiana is a state in the Deep South and South Central regions of the United States. It is the 19th-smallest by area and the 25th most-populous of the 50 U.S. states. Its capital is Baton Rouge, and its largest city is New Orleans.
+[4] ACTION: current_info
+[4] INPUT: {'query': 'Louisiana coastal erosion rate acres per year'}
+[4] OBS: Real-time data for 'Louisiana coastal erosion rate acres per year' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
+FINAL: I was unable to find the annual land loss rate due to coastal erosion in Louisiana. Without that figure, I cannot calculate how much land would be lost over 50 years. My searches returned only general information about Louisiana rather than the specific erosion statistics needed.</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>0b3f5839,b37fb3ed,8ddf9faa</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>SYN_L056_T3</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>TASK: Find the total area of land lost to erosion along the Louisiana coastline each year and calculate how much would be lost in 50 years at that rate.
+[1] ACTION: wikipedia_lookup
+[1] INPUT: {'query': 'Louisiana coastal erosion land loss per year acres'}
+[1] OBS: Page: Louisiana
+Summary: Louisiana is a state in the Deep South and South Central regions of the United States. It is the 19th-smallest by area and the 25th most-populous of the 50 U.S. states. Its capital is Baton Rouge, and its largest city is New Orleans.
+[2] ACTION: wikipedia_lookup
+[2] INPUT: {'query': 'Louisiana coast land erosion rate square miles annually'}
+[2] OBS: Page: Louisiana
+Summary: Louisiana is a state in the Deep South and South Central regions of the United States. It is the 19th-smallest by area and the 25th most-populous of the 50 U.S. states. Its capital is Baton Rouge, and its largest city is New Orleans.
+[3] THOUGHT: I need more specific information about the coastal erosion rate. Let me try a more targeted search.
+[3] ACTION: wikipedia_lookup
+[3] INPUT: {'query': 'Louisiana wetlands coastal erosion land loss rate statistics'}
+[3] OBS: Page: Louisiana
+Summary: Louisiana is a state in the Deep South and South Central regions of the United States. It is the 19th-smallest by area and the 25th most-populous of the 50 U.S. states. Its capital is Baton Rouge, and its largest city is New Orleans.</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_TRUNCATED</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>SYN_L056</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: verifying new loop traces
</commit_message>
<xml_diff>
--- a/loop_augmented_truncated.xlsx
+++ b/loop_augmented_truncated.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J149"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7666,7 +7666,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SYN_L038</t>
+          <t>SYN_L039</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -7680,7 +7680,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
@@ -7690,120 +7690,6 @@
         </is>
       </c>
       <c r="H112" t="inlineStr">
-        <is>
-          <t>TASK: Research the founding members of the Wi-Fi Alliance and compile a summary of each member organisation's current technology portfolio.
-[1] ACTION: wikipedia_lookup
-[1] INPUT: {'query': 'Wi-Fi Alliance founding members organisations'}
-[1] OBS: Page: Wi-Fi Alliance
-Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
-[2] THOUGHT: The article mentions some members but I need the founding members specifically. Let me search more specifically.
-[2] ACTION: wikipedia_lookup
-[2] INPUT: {'query': 'Wi-Fi Alliance founding members 1999 original list'}
-[2] OBS: Page: Wi-Fi Alliance
-Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
-[3] ACTION: wikipedia_lookup
-[3] INPUT: {'query': 'Wi-Fi Alliance history founders founding organisations technology'}
-[3] OBS: Page: Wi-Fi Alliance
-Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
-[4] ACTION: current_info
-[4] INPUT: {'query': 'Wi-Fi Alliance founding member organisations current technology portfolio'}
-[4] OBS: Real-time data for 'Wi-Fi Alliance founding member organisations current technology portfolio' is not available in this system. This system cannot access live stock prices, real-time news, or current market data. For stock purchase tasks: use purchase_mock with a reasonable estimated price and note the real price was unavailable. For weather tasks: use get_weather_mock.
-FINAL: I don't have access to the specific founding members of the Wi-Fi Alliance or their current technology portfolios. The</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J112" t="inlineStr">
-        <is>
-          <t>4b92af45,de469b78,36fdff20</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>SYN_L038_T3</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D113" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>TASK: Research the founding members of the Wi-Fi Alliance and compile a summary of each member organisation's current technology portfolio.
-[1] ACTION: wikipedia_lookup
-[1] INPUT: {'query': 'Wi-Fi Alliance founding members organisations'}
-[1] OBS: Page: Wi-Fi Alliance
-Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
-[2] THOUGHT: The article mentions some members but I need the founding members specifically. Let me search more specifically.
-[2] ACTION: wikipedia_lookup
-[2] INPUT: {'query': 'Wi-Fi Alliance founding members 1999 original list'}
-[2] OBS: Page: Wi-Fi Alliance
-Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.
-[3] ACTION: wikipedia_lookup
-[3] INPUT: {'query': 'Wi-Fi Alliance history founders founding organisations technology'}
-[3] OBS: Page: Wi-Fi Alliance
-Summary: The Wi-Fi Alliance is a non-profit organization that owns the Wi-Fi trademark. Manufacturers may use the trademark to brand products certified for Wi-Fi interoperability. The alliance has more than 800 member companies, including Apple, AT&amp;T, Dell, Ericsson, HP, Intel, Microsoft, Nokia, and Qualcomm.</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>SYNTHETIC_TRUNCATED</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t>SYN_L038</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>SYN_L039</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D114" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
         <is>
           <t>TASK: Who were the original members of the Impressionist movement in painting and what year did they hold their first exhibition?
 [1] THOUGHT: I'll look up the Impressionist movement to find the founding members and their first exhibition date.
@@ -7827,44 +7713,44 @@
 FINAL: I was unable to find specific details about the founding members of the Impressionist movement and the date of their first exhibition. The tools available to me did not return the detailed information required to answer this question.</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J114" t="inlineStr">
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
         <is>
           <t>46b63241,d9c46fce,9d91653a</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
+    <row r="113">
+      <c r="A113" t="inlineStr">
         <is>
           <t>SYN_L039_T3</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D115" t="n">
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
         <v>0.92</v>
       </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr">
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr">
+      <c r="H113" t="inlineStr">
         <is>
           <t>TASK: Who were the original members of the Impressionist movement in painting and what year did they hold their first exhibition?
 [1] THOUGHT: I'll look up the Impressionist movement to find the founding members and their first exhibition date.
@@ -7884,44 +7770,44 @@
 Summary: Impressionism is a 19th-century art movement characterized by relatively small, thin, yet visible brush strokes, open composition, emphasis on accurate depiction of light in its changing qualities, ordinary subject matter, unusual visual angles, and inclusion of movement as a crucial element of human perception and experience.</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr">
+      <c r="I113" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr">
+      <c r="J113" t="inlineStr">
         <is>
           <t>SYN_L039</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
+    <row r="114">
+      <c r="A114" t="inlineStr">
         <is>
           <t>SYN_L040</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D116" t="n">
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
         <v>0.92</v>
       </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr">
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr">
+      <c r="H114" t="inlineStr">
         <is>
           <t>TASK: Find out what instruments were used in the recording of Miles Davis's Kind of Blue and how many tracks the album contains.
 [1] ACTION: wikipedia_lookup
@@ -7948,44 +7834,44 @@
 FINAL: I don't have access to the detailed instrument and track listing information for Kind of Blue. Every search returned only a general summary without the specifics needed to answer the question.</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J116" t="inlineStr">
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
         <is>
           <t>46b63241,d9c46fce,9d91653a</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
+    <row r="115">
+      <c r="A115" t="inlineStr">
         <is>
           <t>SYN_L040_T3</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D117" t="n">
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
         <v>0.92</v>
       </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr"/>
-      <c r="G117" t="inlineStr">
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr">
+      <c r="H115" t="inlineStr">
         <is>
           <t>TASK: Find out what instruments were used in the recording of Miles Davis's Kind of Blue and how many tracks the album contains.
 [1] ACTION: wikipedia_lookup
@@ -8003,44 +7889,44 @@
 Summary: Kind of Blue is a studio album by American jazz musician Miles Davis. It was released on August 17, 1959, by Columbia Records and is widely considered one of the greatest and most influential albums ever made.</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr">
+      <c r="I115" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr">
+      <c r="J115" t="inlineStr">
         <is>
           <t>SYN_L040</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
+    <row r="116">
+      <c r="A116" t="inlineStr">
         <is>
           <t>SYN_L041</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D118" t="n">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
         <v>0.92</v>
       </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
-      <c r="G118" t="inlineStr">
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr">
+      <c r="H116" t="inlineStr">
         <is>
           <t>TASK: What was Frida Kahlo's artistic style and how many self-portraits did she paint in her lifetime?
 [1] ACTION: wikipedia_lookup
@@ -8062,44 +7948,44 @@
 FINAL: I was unable to find the specific number of self-portraits Frida Kahlo painted or a detailed breakdown of her artistic style. The searches returned only a general summary each time.</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J118" t="inlineStr">
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
         <is>
           <t>46b63241,d9c46fce,9d91653a</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
+    <row r="117">
+      <c r="A117" t="inlineStr">
         <is>
           <t>SYN_L041_T3</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D119" t="n">
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
         <v>0.92</v>
       </c>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr">
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr">
+      <c r="H117" t="inlineStr">
         <is>
           <t>TASK: What was Frida Kahlo's artistic style and how many self-portraits did she paint in her lifetime?
 [1] ACTION: wikipedia_lookup
@@ -8117,44 +8003,44 @@
 Summary: Frida Kahlo de Rivera was a Mexican painter known for her many portraits, self-portraits, and works inspired by the nature and artifacts of Mexico. Her work has been celebrated in Mexico as emblematic of national and indigenous tradition and by feminists for its uncompromising depiction of the female experience and form.</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr">
+      <c r="I117" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr">
+      <c r="J117" t="inlineStr">
         <is>
           <t>SYN_L041</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
+    <row r="118">
+      <c r="A118" t="inlineStr">
         <is>
           <t>SYN_L042</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D120" t="n">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
         <v>0.92</v>
       </c>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr">
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr">
+      <c r="H118" t="inlineStr">
         <is>
           <t>TASK: Research the life of composer Johann Sebastian Bach and calculate how many years he lived.
 [1] ACTION: wikipedia_lookup
@@ -8177,44 +8063,44 @@
 FINAL: I was unable to retrieve the specific birth and death dates for Johann Sebastian Bach from the available tools, so I cannot calculate how many years he lived.</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
         <is>
           <t>46b63241,d9c46fce,9d91653a</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
+    <row r="119">
+      <c r="A119" t="inlineStr">
         <is>
           <t>SYN_L042_T3</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D121" t="n">
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
         <v>0.92</v>
       </c>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr">
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr">
+      <c r="H119" t="inlineStr">
         <is>
           <t>TASK: Research the life of composer Johann Sebastian Bach and calculate how many years he lived.
 [1] ACTION: wikipedia_lookup
@@ -8232,44 +8118,44 @@
 Summary: Johann Sebastian Bach was a German composer and musician of the late Baroque period. He is known for instrumental compositions such as the Brandenburg Concertos and the Goldberg Variations, and for vocal music such as the St Matthew Passion and the Mass in B minor.</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr">
+      <c r="I119" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr">
+      <c r="J119" t="inlineStr">
         <is>
           <t>SYN_L042</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
+    <row r="120">
+      <c r="A120" t="inlineStr">
         <is>
           <t>SYN_L043</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D122" t="n">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
         <v>0.97</v>
       </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
-      <c r="G122" t="inlineStr">
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr">
+      <c r="H120" t="inlineStr">
         <is>
           <t>TASK: Find the names of the musicians who performed on The Beatles' Abbey Road album and how many songs are on it.
 [1] ACTION: wikipedia_lookup
@@ -8295,44 +8181,44 @@
 FINAL: I don't have access to the detailed track listing or full personnel information for Abbey Road. Each search returned only the same general album summary without the specifics I needed.</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J122" t="inlineStr">
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
         <is>
           <t>46b63241,d9c46fce,9d91653a</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
+    <row r="121">
+      <c r="A121" t="inlineStr">
         <is>
           <t>SYN_L043_T3</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D123" t="n">
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
         <v>0.97</v>
       </c>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr">
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr">
+      <c r="H121" t="inlineStr">
         <is>
           <t>TASK: Find the names of the musicians who performed on The Beatles' Abbey Road album and how many songs are on it.
 [1] ACTION: wikipedia_lookup
@@ -8350,44 +8236,44 @@
 Summary: Abbey Road is the eleventh studio album by the English rock band the Beatles, released on 26 September 1969 by Apple Records. It is named after the London street where the Beatles' recording studio, Abbey Road Studios, is located.</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr">
+      <c r="I121" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr">
+      <c r="J121" t="inlineStr">
         <is>
           <t>SYN_L043</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
+    <row r="122">
+      <c r="A122" t="inlineStr">
         <is>
           <t>SYN_L044</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D124" t="n">
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
         <v>0.92</v>
       </c>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr">
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 4]</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr">
+      <c r="H122" t="inlineStr">
         <is>
           <t>TASK: What artistic techniques did Leonardo da Vinci use in painting the Mona Lisa?
 [1] THOUGHT: I'll look up the Mona Lisa to find information about the painting techniques Leonardo used.
@@ -8414,44 +8300,44 @@
 FINAL: I was unable to retrieve detailed information about the specific artistic techniques Leonardo da Vinci used in painting the Mona Lisa. The tool searches only returned general summaries of the painting and its artist.</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
         <is>
           <t>46b63241,d9c46fce,9d91653a</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
+    <row r="123">
+      <c r="A123" t="inlineStr">
         <is>
           <t>SYN_L044_T4</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D125" t="n">
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
         <v>0.92</v>
       </c>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr">
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 4]</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr">
+      <c r="H123" t="inlineStr">
         <is>
           <t>TASK: What artistic techniques did Leonardo da Vinci use in painting the Mona Lisa?
 [1] THOUGHT: I'll look up the Mona Lisa to find information about the painting techniques Leonardo used.
@@ -8474,44 +8360,44 @@
 Summary: The Mona Lisa is a half-length portrait painting by Italian artist Leonardo da Vinci. Considered an archetypal masterpiece of the Italian Renaissance, it has been described as "the best known, the most visited, the most written about, the most sung about, the most parodied work of art in the world."</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr">
+      <c r="I123" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr">
+      <c r="J123" t="inlineStr">
         <is>
           <t>SYN_L044</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
+    <row r="124">
+      <c r="A124" t="inlineStr">
         <is>
           <t>SYN_L045</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D126" t="n">
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
         <v>0.97</v>
       </c>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr">
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr">
+      <c r="H124" t="inlineStr">
         <is>
           <t>TASK: Find the distance from Earth to the nearest star outside our solar system and the distance to the center of the Milky Way galaxy, then calculate the ratio between them.
 [1] THOUGHT: I'll start by looking up the distance to the nearest star outside our solar system.
@@ -8536,44 +8422,44 @@
 FINAL: I was unable to find the distance to the nearest star outside our solar system. The tool kept returning the Solar System page without the specific distance data I needed, so I cannot calculate the ratio between the two distances.</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
         <is>
           <t>0efc9456,423d4398,17804dec</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
+    <row r="125">
+      <c r="A125" t="inlineStr">
         <is>
           <t>SYN_L045_T3</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D127" t="n">
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
         <v>0.97</v>
       </c>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr">
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr">
+      <c r="H125" t="inlineStr">
         <is>
           <t>TASK: Find the distance from Earth to the nearest star outside our solar system and the distance to the center of the Milky Way galaxy, then calculate the ratio between them.
 [1] THOUGHT: I'll start by looking up the distance to the nearest star outside our solar system.
@@ -8593,44 +8479,44 @@
 Summary: The Solar System is the gravitationally bound system of the Sun and the objects that orbit it. It formed 4.6 billion years ago from the gravitational collapse of a giant molecular cloud. The vast majority of the system's mass is in the Sun, with most of the remaining mass contained in the planet Jupiter.</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr">
+      <c r="I125" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr">
+      <c r="J125" t="inlineStr">
         <is>
           <t>SYN_L045</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
+    <row r="126">
+      <c r="A126" t="inlineStr">
         <is>
           <t>SYN_L046</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D128" t="n">
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
         <v>0.92</v>
       </c>
-      <c r="E128" t="inlineStr"/>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr">
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 5]</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr">
+      <c r="H126" t="inlineStr">
         <is>
           <t>TASK: What is the surface temperature of Venus and the surface temperature of Mars? Calculate how many times hotter Venus is than Mars.
 [1] ACTION: wikipedia_lookup
@@ -8658,44 +8544,44 @@
 FINAL: I was unable to retrieve the specific surface temperatures of Venus or Mars from the available tool. The Wikipedia summaries returned only general descriptions without the numerical temperature values I needed to perform the calculation.</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
         <is>
           <t>0efc9456,423d4398,17804dec</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
+    <row r="127">
+      <c r="A127" t="inlineStr">
         <is>
           <t>SYN_L046_T5</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D129" t="n">
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
         <v>0.92</v>
       </c>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr">
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 5]</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr">
+      <c r="H127" t="inlineStr">
         <is>
           <t>TASK: What is the surface temperature of Venus and the surface temperature of Mars? Calculate how many times hotter Venus is than Mars.
 [1] ACTION: wikipedia_lookup
@@ -8722,44 +8608,44 @@
 Summary: Venus is the second planet from the Sun. It is a terrestrial planet and is the closest in mass and size to its orbital neighbour Earth. Venus has by far the densest atmosphere of the terrestrial planets, composed mostly of carbon dioxide with a thick, global sulfuric acid cloud cover. The planet is named after and associated with the Roman goddess of love and beauty.</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr">
+      <c r="I127" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr">
+      <c r="J127" t="inlineStr">
         <is>
           <t>SYN_L046</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
+    <row r="128">
+      <c r="A128" t="inlineStr">
         <is>
           <t>SYN_L047</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D130" t="n">
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
         <v>0.92</v>
       </c>
-      <c r="E130" t="inlineStr"/>
-      <c r="F130" t="inlineStr"/>
-      <c r="G130" t="inlineStr">
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr">
+      <c r="H128" t="inlineStr">
         <is>
           <t>TASK: Find the orbital period of Jupiter and the orbital period of Saturn, then calculate how much longer Saturn's year is compared to Jupiter's.
 [1] ACTION: wikipedia_lookup
@@ -8789,44 +8675,44 @@
 FINAL: I was unable to find the specific orbital periods for Jupiter and Saturn. Both the Wikipedia summaries and current_info tool failed to return the numerical data needed to calculate the difference between Saturn's and Jupiter's orbital periods.</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J130" t="inlineStr">
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
         <is>
           <t>0efc9456,423d4398,17804dec</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
+    <row r="129">
+      <c r="A129" t="inlineStr">
         <is>
           <t>SYN_L047_T3</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D131" t="n">
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
         <v>0.92</v>
       </c>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr">
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr">
+      <c r="H129" t="inlineStr">
         <is>
           <t>TASK: Find the orbital period of Jupiter and the orbital period of Saturn, then calculate how much longer Saturn's year is compared to Jupiter's.
 [1] ACTION: wikipedia_lookup
@@ -8844,44 +8730,44 @@
 Summary: Jupiter is the fifth planet from the Sun and the largest in the Solar System. It is a gas giant with a mass more than 2.5 times that of all the other planets in the Solar System combined, and slightly less than one-thousandth the mass of the Sun. Jupiter is the third brightest natural object in the night sky after the Moon and Venus, and has been observed since prehistoric times.</t>
         </is>
       </c>
-      <c r="I131" t="inlineStr">
+      <c r="I129" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr">
+      <c r="J129" t="inlineStr">
         <is>
           <t>SYN_L047</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
+    <row r="130">
+      <c r="A130" t="inlineStr">
         <is>
           <t>SYN_L048</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D132" t="n">
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
         <v>0.92</v>
       </c>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr">
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr">
+      <c r="H130" t="inlineStr">
         <is>
           <t>TASK: Look up the diameter of the Andromeda Galaxy and the diameter of the Milky Way and find the percentage difference between them.
 [1] ACTION: wikipedia_lookup
@@ -8905,44 +8791,44 @@
 FINAL: I was unable to retrieve the specific diameter values for either the Andromeda Galaxy or the Milky Way. The Wikipedia summaries returned general descriptions without the numerical measurements needed to calculate a percentage difference.</t>
         </is>
       </c>
-      <c r="I132" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J132" t="inlineStr">
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
         <is>
           <t>0efc9456,423d4398,17804dec</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
+    <row r="131">
+      <c r="A131" t="inlineStr">
         <is>
           <t>SYN_L048_T3</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D133" t="n">
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
         <v>0.92</v>
       </c>
-      <c r="E133" t="inlineStr"/>
-      <c r="F133" t="inlineStr"/>
-      <c r="G133" t="inlineStr">
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr">
+      <c r="H131" t="inlineStr">
         <is>
           <t>TASK: Look up the diameter of the Andromeda Galaxy and the diameter of the Milky Way and find the percentage difference between them.
 [1] ACTION: wikipedia_lookup
@@ -8961,44 +8847,44 @@
 Summary: The Andromeda Galaxy, also known as Messier 31, is a barred spiral galaxy and is the nearest major galaxy to the Milky Way. It was named after the princess Andromeda in Greek mythology. Andromeda is the largest galaxy of the Local Group, which also contains the Milky Way, the Triangulum Galaxy, and about 54 other smaller galaxies.</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr">
+      <c r="I131" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr">
+      <c r="J131" t="inlineStr">
         <is>
           <t>SYN_L048</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
+    <row r="132">
+      <c r="A132" t="inlineStr">
         <is>
           <t>SYN_L049</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D134" t="n">
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
         <v>0.92</v>
       </c>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr"/>
-      <c r="G134" t="inlineStr">
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 3, 5]</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr">
+      <c r="H132" t="inlineStr">
         <is>
           <t>TASK: What is the mass of the Sun compared to the mass of the Earth? Find both values and compute the ratio.
 [1] ACTION: wikipedia_lookup
@@ -9025,44 +8911,44 @@
 FINAL: I don't have access to the specific mass values for the Sun and Earth. Each query returned only general summary paragraphs without numerical data, making it impossible to compute the ratio between them.</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J134" t="inlineStr">
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
         <is>
           <t>0efc9456,423d4398,17804dec</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
+    <row r="133">
+      <c r="A133" t="inlineStr">
         <is>
           <t>SYN_L049_T5</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D135" t="n">
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
         <v>0.92</v>
       </c>
-      <c r="E135" t="inlineStr"/>
-      <c r="F135" t="inlineStr"/>
-      <c r="G135" t="inlineStr">
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 3, 5]</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr">
+      <c r="H133" t="inlineStr">
         <is>
           <t>TASK: What is the mass of the Sun compared to the mass of the Earth? Find both values and compute the ratio.
 [1] ACTION: wikipedia_lookup
@@ -9088,44 +8974,44 @@
 Summary: The Sun is the star at the center of the Solar System. It is a massive, nearly perfect sphere of hot plasma, heated to incandescence by nuclear fusion reactions in its core. The Sun radiates this energy mainly as light, ultraviolet, and infrared radiation, and is the most important source of energy for life on Earth.</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr">
+      <c r="I133" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr">
+      <c r="J133" t="inlineStr">
         <is>
           <t>SYN_L049</t>
         </is>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
+    <row r="134">
+      <c r="A134" t="inlineStr">
         <is>
           <t>SYN_L050</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D136" t="n">
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
         <v>0.9</v>
       </c>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr">
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr">
+      <c r="H134" t="inlineStr">
         <is>
           <t>TASK: Find how long it takes light to travel from the Sun to Neptune and from the Sun to Pluto, and calculate the difference in travel time.
 [1] THOUGHT: I'll look up the distance from the Sun to Neptune first, then to Pluto, and use the speed of light to compute travel times.
@@ -9152,44 +9038,44 @@
 FINAL: I was unable to find the specific distances from the Sun to Neptune and Pluto. Without those values, I cannot calculate the light travel times or the difference between them.</t>
         </is>
       </c>
-      <c r="I136" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J136" t="inlineStr">
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
         <is>
           <t>0efc9456,423d4398,17804dec</t>
         </is>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
+    <row r="135">
+      <c r="A135" t="inlineStr">
         <is>
           <t>SYN_L050_T3</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D137" t="n">
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
         <v>0.9</v>
       </c>
-      <c r="E137" t="inlineStr"/>
-      <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr">
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr">
+      <c r="H135" t="inlineStr">
         <is>
           <t>TASK: Find how long it takes light to travel from the Sun to Neptune and from the Sun to Pluto, and calculate the difference in travel time.
 [1] THOUGHT: I'll look up the distance from the Sun to Neptune first, then to Pluto, and use the speed of light to compute travel times.
@@ -9208,44 +9094,44 @@
 Summary: Neptune is the eighth and farthest known planet from the Sun. It is the fourth-largest planet in the Solar System by diameter, the third-most-massive planet, and the densest giant planet. It is 17 times the mass of Earth.</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr">
+      <c r="I135" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr">
+      <c r="J135" t="inlineStr">
         <is>
           <t>SYN_L050</t>
         </is>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
+    <row r="136">
+      <c r="A136" t="inlineStr">
         <is>
           <t>SYN_L051</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D138" t="n">
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
         <v>0.97</v>
       </c>
-      <c r="E138" t="inlineStr"/>
-      <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr">
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr">
+      <c r="H136" t="inlineStr">
         <is>
           <t>TASK: Find the magnitude of the largest earthquake ever recorded and where it occurred.
 [1] ACTION: wikipedia_lookup
@@ -9264,44 +9150,44 @@
 FINAL: I was unable to find the specific magnitude and location of the largest earthquake ever recorded. The search results kept returning only a general overview page without the specific details needed.</t>
         </is>
       </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
         <is>
           <t>0b3f5839,b37fb3ed,8ddf9faa</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
+    <row r="137">
+      <c r="A137" t="inlineStr">
         <is>
           <t>SYN_L051_T3</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D139" t="n">
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
         <v>0.97</v>
       </c>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
-      <c r="G139" t="inlineStr">
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr">
+      <c r="H137" t="inlineStr">
         <is>
           <t>TASK: Find the magnitude of the largest earthquake ever recorded and where it occurred.
 [1] ACTION: wikipedia_lookup
@@ -9319,44 +9205,44 @@
 Summary: This article lists notable earthquakes that have been recorded historically. Earthquakes are measured using seismometers and the magnitude is calculated using various scales including the Richter scale and moment magnitude scale. The list includes earthquakes that caused significant damage or casualties throughout history.</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr">
+      <c r="I137" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr">
+      <c r="J137" t="inlineStr">
         <is>
           <t>SYN_L051</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
+    <row r="138">
+      <c r="A138" t="inlineStr">
         <is>
           <t>SYN_L052</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D140" t="n">
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
         <v>0.85</v>
       </c>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr">
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr">
+      <c r="H138" t="inlineStr">
         <is>
           <t>TASK: Find the depth of the Mariana Trench and the depth of the Tonga Trench and determine which is deeper and by how many meters.
 [1] ACTION: wikipedia_lookup
@@ -9386,44 +9272,44 @@
 FINAL: I don't have access to the specific depth measurements for the Mariana Trench and the Tonga Trench. I was unable to retrieve the numerical depth values needed to compare the two trenches.</t>
         </is>
       </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
         <is>
           <t>0b3f5839,b37fb3ed,8ddf9faa</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
+    <row r="139">
+      <c r="A139" t="inlineStr">
         <is>
           <t>SYN_L052_T3</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D141" t="n">
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
         <v>0.85</v>
       </c>
-      <c r="E141" t="inlineStr"/>
-      <c r="F141" t="inlineStr"/>
-      <c r="G141" t="inlineStr">
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 4]</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr">
+      <c r="H139" t="inlineStr">
         <is>
           <t>TASK: Find the depth of the Mariana Trench and the depth of the Tonga Trench and determine which is deeper and by how many meters.
 [1] ACTION: wikipedia_lookup
@@ -9441,44 +9327,44 @@
 Summary: The Mariana Trench is an oceanic trench located in the western Pacific Ocean, east of the Mariana Islands. It is the deepest oceanic trench on Earth. The trench is roughly crescent-shaped and measures about 2,550 km in length and 69 km in width.</t>
         </is>
       </c>
-      <c r="I141" t="inlineStr">
+      <c r="I139" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr">
+      <c r="J139" t="inlineStr">
         <is>
           <t>SYN_L052</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
+    <row r="140">
+      <c r="A140" t="inlineStr">
         <is>
           <t>SYN_L053</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D142" t="n">
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
         <v>0.97</v>
       </c>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
-      <c r="G142" t="inlineStr">
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 4]</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr">
+      <c r="H140" t="inlineStr">
         <is>
           <t>TASK: Find how many people were killed in the 1980 Mount St. Helens eruption and how much ash was produced.
 [1] ACTION: wikipedia_lookup
@@ -9501,44 +9387,44 @@
 FINAL: I was unable to find the specific death toll and ash production figures for the 1980 Mount St. Helens eruption. All my searches returned only general information about the volcano without the specific statistics I needed.</t>
         </is>
       </c>
-      <c r="I142" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J142" t="inlineStr">
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
         <is>
           <t>0b3f5839,b37fb3ed,8ddf9faa</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
+    <row r="141">
+      <c r="A141" t="inlineStr">
         <is>
           <t>SYN_L053_T4</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D143" t="n">
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
         <v>0.97</v>
       </c>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr">
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[2, 3, 4]</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr">
+      <c r="H141" t="inlineStr">
         <is>
           <t>TASK: Find how many people were killed in the 1980 Mount St. Helens eruption and how much ash was produced.
 [1] ACTION: wikipedia_lookup
@@ -9560,44 +9446,44 @@
 Summary: Mount St. Helens is a lava dome volcano located in Skamania County, Washington, in the Pacific Northwest region of the United States. It is 154 km south of Seattle and 85 km northeast of Portland, Oregon. The mountain is part of the Cascade Range and is the most active volcano in the contiguous United States.</t>
         </is>
       </c>
-      <c r="I143" t="inlineStr">
+      <c r="I141" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr">
+      <c r="J141" t="inlineStr">
         <is>
           <t>SYN_L053</t>
         </is>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
+    <row r="142">
+      <c r="A142" t="inlineStr">
         <is>
           <t>SYN_L054</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D144" t="n">
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
         <v>0.95</v>
       </c>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
-      <c r="G144" t="inlineStr">
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr">
+      <c r="H142" t="inlineStr">
         <is>
           <t>TASK: Find the date and location of the 2004 Indian Ocean tsunami and how many countries were affected.
 [1] ACTION: wikipedia_lookup
@@ -9619,44 +9505,44 @@
 FINAL: I was unable to find the specific details about the 2004 Indian Ocean tsunami, including the number of countries affected. My searches repeatedly returned general information about the Indian Ocean rather than the tsunami event itself.</t>
         </is>
       </c>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J144" t="inlineStr">
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
         <is>
           <t>0b3f5839,b37fb3ed,8ddf9faa</t>
         </is>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
+    <row r="143">
+      <c r="A143" t="inlineStr">
         <is>
           <t>SYN_L054_T3</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D145" t="n">
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
         <v>0.95</v>
       </c>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr">
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr">
+      <c r="H143" t="inlineStr">
         <is>
           <t>TASK: Find the date and location of the 2004 Indian Ocean tsunami and how many countries were affected.
 [1] ACTION: wikipedia_lookup
@@ -9674,44 +9560,44 @@
 Summary: The Indian Ocean is the third-largest of the world's five oceanic divisions, covering an area of 70,560,000 km2. It is bounded by Asia to the north, Africa to the west, and Australia to the east. To the south it is bounded by the Southern Ocean or Antarctica, depending on the definition used.</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr">
+      <c r="I143" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr">
+      <c r="J143" t="inlineStr">
         <is>
           <t>SYN_L054</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
+    <row r="144">
+      <c r="A144" t="inlineStr">
         <is>
           <t>SYN_L055</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D146" t="n">
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
         <v>0.95</v>
       </c>
-      <c r="E146" t="inlineStr"/>
-      <c r="F146" t="inlineStr"/>
-      <c r="G146" t="inlineStr">
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr">
+      <c r="H144" t="inlineStr">
         <is>
           <t>TASK: Find the flow rate of lava during the 2018 Kilauea eruption in Hawaii and how many homes were destroyed.
 [1] ACTION: wikipedia_lookup
@@ -9738,44 +9624,44 @@
 FINAL: I don't have access to the specific statistics for the 2018 Kilauea eruption. My repeated searches only returned general information about the Kilauea volcano and I was unable to find the lava flow rate or the number of homes destroyed.</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr">
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
         <is>
           <t>0b3f5839,b37fb3ed,8ddf9faa</t>
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
+    <row r="145">
+      <c r="A145" t="inlineStr">
         <is>
           <t>SYN_L055_T3</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
         <v>0.95</v>
       </c>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr">
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3, 5]</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr">
+      <c r="H145" t="inlineStr">
         <is>
           <t>TASK: Find the flow rate of lava during the 2018 Kilauea eruption in Hawaii and how many homes were destroyed.
 [1] ACTION: wikipedia_lookup
@@ -9793,44 +9679,44 @@
 Summary: Kīlauea is a currently active shield volcano in the Hawaiian Islands, and the most active of the five volcanoes that together form the island of Hawaiʻi. Located along the southeastern shore of the island, the volcano is between 210,000 and 280,000 years old.</t>
         </is>
       </c>
-      <c r="I147" t="inlineStr">
+      <c r="I145" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J147" t="inlineStr">
+      <c r="J145" t="inlineStr">
         <is>
           <t>SYN_L055</t>
         </is>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
+    <row r="146">
+      <c r="A146" t="inlineStr">
         <is>
           <t>SYN_L056</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D148" t="n">
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
         <v>0.92</v>
       </c>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr">
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr">
+      <c r="H146" t="inlineStr">
         <is>
           <t>TASK: Find the total area of land lost to erosion along the Louisiana coastline each year and calculate how much would be lost in 50 years at that rate.
 [1] ACTION: wikipedia_lookup
@@ -9852,44 +9738,44 @@
 FINAL: I was unable to find the annual land loss rate due to coastal erosion in Louisiana. Without that figure, I cannot calculate how much land would be lost over 50 years. My searches returned only general information about Louisiana rather than the specific erosion statistics needed.</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
         <is>
           <t>0b3f5839,b37fb3ed,8ddf9faa</t>
         </is>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
+    <row r="147">
+      <c r="A147" t="inlineStr">
         <is>
           <t>SYN_L056_T3</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>LOOP</t>
-        </is>
-      </c>
-      <c r="D149" t="n">
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
         <v>0.92</v>
       </c>
-      <c r="E149" t="inlineStr"/>
-      <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr">
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr">
         <is>
           <t>LLM-generated (round 2), QA-passed via auto-labeller; repeat_steps=[1, 2, 3]</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr">
+      <c r="H147" t="inlineStr">
         <is>
           <t>TASK: Find the total area of land lost to erosion along the Louisiana coastline each year and calculate how much would be lost in 50 years at that rate.
 [1] ACTION: wikipedia_lookup
@@ -9907,12 +9793,12 @@
 Summary: Louisiana is a state in the Deep South and South Central regions of the United States. It is the 19th-smallest by area and the 25th most-populous of the 50 U.S. states. Its capital is Baton Rouge, and its largest city is New Orleans.</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr">
+      <c r="I147" t="inlineStr">
         <is>
           <t>SYNTHETIC_TRUNCATED</t>
         </is>
       </c>
-      <c r="J149" t="inlineStr">
+      <c r="J147" t="inlineStr">
         <is>
           <t>SYN_L056</t>
         </is>

</xml_diff>